<commit_message>
E05: DSCR shown as a multiple, guarded against rounding; rebuilt sample
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ss1SkSGdT4RqYLjEdbFgGp
</commit_message>
<xml_diff>
--- a/samples/real_estate-full.xlsx
+++ b/samples/real_estate-full.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="282">
   <si>
     <t xml:space="preserve">Rental property financial model (early)</t>
   </si>
@@ -693,6 +693,12 @@
     <t xml:space="preserve">Cash-on-cash return (levered cash flow before sale ÷ equity invested)</t>
   </si>
   <si>
+    <t xml:space="preserve">Helper: sign of the unlevered cash flow (a zero keeps the previous sign)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helper: sign of the levered cash flow (a zero keeps the previous sign)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sale at the end of year 3</t>
   </si>
   <si>
@@ -732,6 +738,9 @@
     <t xml:space="preserve">Helper: IRR starting estimate ((inflows ÷ outflows) ^ (1 ÷ years) − 1)</t>
   </si>
   <si>
+    <t xml:space="preserve">Helper: IRR defined (1 = one sign change and inflows ≥ 25% of outflows)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Discount rate for NPV</t>
   </si>
   <si>
@@ -747,7 +756,7 @@
     <t xml:space="preserve">Going-in cap rate (year-1 NOI ÷ purchase price)</t>
   </si>
   <si>
-    <t xml:space="preserve">IRR and NPV use yearly flows with the purchase at year 0 and the sale at the end of the final year. n/a = no debt service, no equity invested, or no IRR exists for these flows.</t>
+    <t xml:space="preserve">IRR and NPV use yearly flows with the purchase at year 0 and the sale at the end of the final year. n/a = no debt service or no equity invested; IRR n/a = the flows change sign more than once (IRR not unique) or return less than 25% of the money put in.</t>
   </si>
   <si>
     <t xml:space="preserve">Live formulas: they re-run every time an input changes.</t>
@@ -871,7 +880,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\-"/>
@@ -879,8 +888,9 @@
     <numFmt numFmtId="168" formatCode="0"/>
     <numFmt numFmtId="169" formatCode="@"/>
     <numFmt numFmtId="170" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="171" formatCode="#,##0;\(#,##0\);\-"/>
-    <numFmt numFmtId="172" formatCode="0.00\x"/>
+    <numFmt numFmtId="171" formatCode="0.0\x"/>
+    <numFmt numFmtId="172" formatCode="#,##0;\(#,##0\);\-"/>
+    <numFmt numFmtId="173" formatCode="0.00\x"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -1080,7 +1090,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1165,6 +1175,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1185,11 +1199,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1209,7 +1223,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1225,7 +1239,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1940,16 +1954,16 @@
       <c r="A38" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="13" t="n">
-        <f aca="false">IF(B37&gt;0,B32/B37,"n/a")</f>
+      <c r="B38" s="21" t="n">
+        <f aca="false">IF(B37&gt;0.5,B32/B37,"n/a")</f>
         <v>1.37709334172061</v>
       </c>
-      <c r="C38" s="13" t="n">
-        <f aca="false">IF(C37&gt;0,C32/C37,"n/a")</f>
+      <c r="C38" s="21" t="n">
+        <f aca="false">IF(C37&gt;0.5,C32/C37,"n/a")</f>
         <v>1.41840614197223</v>
       </c>
-      <c r="D38" s="13" t="n">
-        <f aca="false">IF(D37&gt;0,D32/D37,"n/a")</f>
+      <c r="D38" s="21" t="n">
+        <f aca="false">IF(D37&gt;0.5,D32/D37,"n/a")</f>
         <v>1.4609583262314</v>
       </c>
     </row>
@@ -2034,7 +2048,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="22" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="9" t="s">
@@ -2049,10 +2063,10 @@
       <c r="E5" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="21" t="s">
+      <c r="F5" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="21" t="s">
+      <c r="G5" s="22" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2071,20 +2085,20 @@
       <c r="A7" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>1850000</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>1850000</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>1850000</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B7,C7,D7)</f>
         <v>1850000</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G7" s="17"/>
@@ -2093,20 +2107,20 @@
       <c r="A8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="25" t="n">
         <v>0.2</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="25" t="n">
         <v>0.2</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="25" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B8,C8,D8)</f>
         <v>0.2</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G8" s="17"/>
@@ -2115,20 +2129,20 @@
       <c r="A9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B9,C9,D9)</f>
         <v>0.03</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G9" s="17" t="s">
@@ -2139,20 +2153,20 @@
       <c r="A10" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="28" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B10,C10,D10)</f>
         <v>10</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="24" t="s">
         <v>53</v>
       </c>
       <c r="G10" s="17"/>
@@ -2172,20 +2186,20 @@
       <c r="A13" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="28" t="n">
+      <c r="B13" s="29" t="n">
         <v>1600</v>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="29" t="n">
         <v>1700</v>
       </c>
-      <c r="D13" s="28" t="n">
+      <c r="D13" s="29" t="n">
         <v>1800</v>
       </c>
-      <c r="E13" s="29" t="n">
+      <c r="E13" s="30" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B13,C13,D13)</f>
         <v>1700</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G13" s="17" t="s">
@@ -2196,20 +2210,20 @@
       <c r="A14" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="25" t="n">
         <v>0.02</v>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="25" t="n">
         <v>0.04</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B14,C14,D14)</f>
         <v>0.03</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G14" s="17" t="s">
@@ -2220,20 +2234,20 @@
       <c r="A15" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="25" t="n">
         <v>0.08</v>
       </c>
-      <c r="C15" s="24" t="n">
+      <c r="C15" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="25" t="n">
         <v>0.04</v>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E15" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B15,C15,D15)</f>
         <v>0.05</v>
       </c>
-      <c r="F15" s="23" t="s">
+      <c r="F15" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G15" s="17" t="s">
@@ -2244,20 +2258,20 @@
       <c r="A16" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="28" t="n">
+      <c r="B16" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="29" t="n">
         <v>25</v>
       </c>
-      <c r="D16" s="28" t="n">
+      <c r="D16" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="E16" s="29" t="n">
+      <c r="E16" s="30" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B16,C16,D16)</f>
         <v>25</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="F16" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G16" s="17" t="s">
@@ -2279,20 +2293,20 @@
       <c r="A19" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="25" t="n">
         <v>0.07</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="25" t="n">
         <v>0.06</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="E19" s="25" t="n">
+      <c r="E19" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B19,C19,D19)</f>
         <v>0.06</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G19" s="17" t="s">
@@ -2303,20 +2317,20 @@
       <c r="A20" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="22" t="n">
+      <c r="B20" s="23" t="n">
         <v>900</v>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C20" s="23" t="n">
         <v>900</v>
       </c>
-      <c r="D20" s="22" t="n">
+      <c r="D20" s="23" t="n">
         <v>900</v>
       </c>
       <c r="E20" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B20,C20,D20)</f>
         <v>900</v>
       </c>
-      <c r="F20" s="23" t="s">
+      <c r="F20" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G20" s="17"/>
@@ -2325,20 +2339,20 @@
       <c r="A21" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="24" t="n">
+      <c r="B21" s="25" t="n">
         <v>0.011</v>
       </c>
-      <c r="C21" s="24" t="n">
+      <c r="C21" s="25" t="n">
         <v>0.011</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="25" t="n">
         <v>0.011</v>
       </c>
-      <c r="E21" s="25" t="n">
+      <c r="E21" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B21,C21,D21)</f>
         <v>0.011</v>
       </c>
-      <c r="F21" s="23" t="s">
+      <c r="F21" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G21" s="17"/>
@@ -2347,20 +2361,20 @@
       <c r="A22" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="22" t="n">
+      <c r="B22" s="23" t="n">
         <v>800</v>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="23" t="n">
         <v>800</v>
       </c>
-      <c r="D22" s="22" t="n">
+      <c r="D22" s="23" t="n">
         <v>800</v>
       </c>
       <c r="E22" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B22,C22,D22)</f>
         <v>800</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="F22" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G22" s="17"/>
@@ -2369,20 +2383,20 @@
       <c r="A23" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="24" t="n">
+      <c r="B23" s="25" t="n">
         <v>0.08</v>
       </c>
-      <c r="C23" s="24" t="n">
+      <c r="C23" s="25" t="n">
         <v>0.08</v>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="25" t="n">
         <v>0.08</v>
       </c>
-      <c r="E23" s="25" t="n">
+      <c r="E23" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B23,C23,D23)</f>
         <v>0.08</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G23" s="17" t="s">
@@ -2393,20 +2407,20 @@
       <c r="A24" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="22" t="n">
+      <c r="B24" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C24" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="D24" s="22" t="n">
+      <c r="D24" s="23" t="n">
         <v>400</v>
       </c>
       <c r="E24" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B24,C24,D24)</f>
         <v>400</v>
       </c>
-      <c r="F24" s="23" t="s">
+      <c r="F24" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G24" s="17"/>
@@ -2415,20 +2429,20 @@
       <c r="A25" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="24" t="n">
+      <c r="B25" s="25" t="n">
         <v>0.04</v>
       </c>
-      <c r="C25" s="24" t="n">
+      <c r="C25" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="D25" s="24" t="n">
+      <c r="D25" s="25" t="n">
         <v>0.025</v>
       </c>
-      <c r="E25" s="25" t="n">
+      <c r="E25" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B25,C25,D25)</f>
         <v>0.03</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="F25" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G25" s="17" t="s">
@@ -2439,20 +2453,20 @@
       <c r="A26" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="22" t="n">
+      <c r="B26" s="23" t="n">
         <v>350</v>
       </c>
-      <c r="C26" s="22" t="n">
+      <c r="C26" s="23" t="n">
         <v>350</v>
       </c>
-      <c r="D26" s="22" t="n">
+      <c r="D26" s="23" t="n">
         <v>350</v>
       </c>
       <c r="E26" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B26,C26,D26)</f>
         <v>350</v>
       </c>
-      <c r="F26" s="23" t="s">
+      <c r="F26" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G26" s="17"/>
@@ -2472,20 +2486,20 @@
       <c r="A29" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="24" t="n">
+      <c r="B29" s="25" t="n">
         <v>0.0725</v>
       </c>
-      <c r="C29" s="24" t="n">
+      <c r="C29" s="25" t="n">
         <v>0.0675</v>
       </c>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="25" t="n">
         <v>0.0625</v>
       </c>
-      <c r="E29" s="25" t="n">
+      <c r="E29" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B29,C29,D29)</f>
         <v>0.0675</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G29" s="17" t="s">
@@ -2496,20 +2510,20 @@
       <c r="A30" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="24" t="n">
+      <c r="B30" s="25" t="n">
         <v>0.06</v>
       </c>
-      <c r="C30" s="24" t="n">
+      <c r="C30" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="D30" s="24" t="n">
+      <c r="D30" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="E30" s="25" t="n">
+      <c r="E30" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B30,C30,D30)</f>
         <v>0.05</v>
       </c>
-      <c r="F30" s="23" t="s">
+      <c r="F30" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G30" s="17" t="s">
@@ -2520,20 +2534,20 @@
       <c r="A31" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="24" t="n">
+      <c r="B31" s="25" t="n">
         <v>0.1</v>
       </c>
-      <c r="C31" s="24" t="n">
+      <c r="C31" s="25" t="n">
         <v>0.1</v>
       </c>
-      <c r="D31" s="24" t="n">
+      <c r="D31" s="25" t="n">
         <v>0.1</v>
       </c>
-      <c r="E31" s="25" t="n">
+      <c r="E31" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B31,C31,D31)</f>
         <v>0.1</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="F31" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G31" s="17"/>
@@ -2553,20 +2567,20 @@
       <c r="A34" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B34" s="22" t="n">
+      <c r="B34" s="23" t="n">
         <v>760000</v>
       </c>
-      <c r="C34" s="22" t="n">
+      <c r="C34" s="23" t="n">
         <v>760000</v>
       </c>
-      <c r="D34" s="22" t="n">
+      <c r="D34" s="23" t="n">
         <v>760000</v>
       </c>
       <c r="E34" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B34,C34,D34)</f>
         <v>760000</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="F34" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G34" s="17"/>
@@ -2575,20 +2589,20 @@
       <c r="A35" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="22" t="n">
+      <c r="B35" s="23" t="n">
         <v>1200000</v>
       </c>
-      <c r="C35" s="22" t="n">
+      <c r="C35" s="23" t="n">
         <v>1200000</v>
       </c>
-      <c r="D35" s="22" t="n">
+      <c r="D35" s="23" t="n">
         <v>1200000</v>
       </c>
       <c r="E35" s="15" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B35,C35,D35)</f>
         <v>1200000</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="F35" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G35" s="17"/>
@@ -2597,20 +2611,20 @@
       <c r="A36" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B36" s="24" t="n">
+      <c r="B36" s="25" t="n">
         <v>0.065</v>
       </c>
-      <c r="C36" s="24" t="n">
+      <c r="C36" s="25" t="n">
         <v>0.065</v>
       </c>
-      <c r="D36" s="24" t="n">
+      <c r="D36" s="25" t="n">
         <v>0.065</v>
       </c>
-      <c r="E36" s="25" t="n">
+      <c r="E36" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B36,C36,D36)</f>
         <v>0.065</v>
       </c>
-      <c r="F36" s="23" t="s">
+      <c r="F36" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G36" s="17"/>
@@ -2619,20 +2633,20 @@
       <c r="A37" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="26" t="n">
+      <c r="B37" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="C37" s="26" t="n">
+      <c r="C37" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="D37" s="26" t="n">
+      <c r="D37" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="E37" s="27" t="n">
+      <c r="E37" s="28" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B37,C37,D37)</f>
         <v>30</v>
       </c>
-      <c r="F37" s="23" t="s">
+      <c r="F37" s="24" t="s">
         <v>78</v>
       </c>
       <c r="G37" s="17"/>
@@ -2652,20 +2666,20 @@
       <c r="A40" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="B40" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="27" t="n">
+      <c r="B40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="28" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B40,C40,D40)</f>
         <v>0</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" s="24" t="s">
         <v>81</v>
       </c>
       <c r="G40" s="17"/>
@@ -2674,20 +2688,20 @@
       <c r="A41" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B41" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="C41" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="27" t="n">
+      <c r="B41" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="28" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B41,C41,D41)</f>
         <v>0</v>
       </c>
-      <c r="F41" s="23" t="s">
+      <c r="F41" s="24" t="s">
         <v>81</v>
       </c>
       <c r="G41" s="17"/>
@@ -2696,20 +2710,20 @@
       <c r="A42" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B42" s="26" t="n">
+      <c r="B42" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="C42" s="26" t="n">
+      <c r="C42" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="D42" s="26" t="n">
+      <c r="D42" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="E42" s="27" t="n">
+      <c r="E42" s="28" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B42,C42,D42)</f>
         <v>15</v>
       </c>
-      <c r="F42" s="23" t="s">
+      <c r="F42" s="24" t="s">
         <v>81</v>
       </c>
       <c r="G42" s="17"/>
@@ -2729,20 +2743,20 @@
       <c r="A45" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B45" s="26" t="n">
+      <c r="B45" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="C45" s="26" t="n">
+      <c r="C45" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="D45" s="26" t="n">
+      <c r="D45" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="E45" s="27" t="n">
+      <c r="E45" s="28" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B45,C45,D45)</f>
         <v>27</v>
       </c>
-      <c r="F45" s="23" t="s">
+      <c r="F45" s="24" t="s">
         <v>78</v>
       </c>
       <c r="G45" s="17"/>
@@ -2751,20 +2765,20 @@
       <c r="A46" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B46" s="24" t="n">
+      <c r="B46" s="25" t="n">
         <v>0.21</v>
       </c>
-      <c r="C46" s="24" t="n">
+      <c r="C46" s="25" t="n">
         <v>0.21</v>
       </c>
-      <c r="D46" s="24" t="n">
+      <c r="D46" s="25" t="n">
         <v>0.21</v>
       </c>
-      <c r="E46" s="25" t="n">
+      <c r="E46" s="26" t="n">
         <f aca="false">CHOOSE(Dashboard!$B$4,B46,C46,D46)</f>
         <v>0.21</v>
       </c>
-      <c r="F46" s="23" t="s">
+      <c r="F46" s="24" t="s">
         <v>49</v>
       </c>
       <c r="G46" s="17"/>
@@ -2940,112 +2954,112 @@
       <c r="A4" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="C4" s="30" t="n">
+      <c r="C4" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="30" t="n">
+      <c r="D4" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="30" t="n">
+      <c r="E4" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="30" t="n">
+      <c r="F4" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="30" t="n">
+      <c r="G4" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="30" t="n">
+      <c r="H4" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="30" t="n">
+      <c r="I4" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="30" t="n">
+      <c r="J4" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="K4" s="30" t="n">
+      <c r="K4" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="L4" s="30" t="n">
+      <c r="L4" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="M4" s="30" t="n">
+      <c r="M4" s="31" t="n">
         <v>11</v>
       </c>
-      <c r="N4" s="30" t="n">
+      <c r="N4" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="O4" s="30" t="n">
+      <c r="O4" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="P4" s="30" t="n">
+      <c r="P4" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="Q4" s="30" t="n">
+      <c r="Q4" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="R4" s="30" t="n">
+      <c r="R4" s="31" t="n">
         <v>16</v>
       </c>
-      <c r="S4" s="30" t="n">
+      <c r="S4" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="T4" s="30" t="n">
+      <c r="T4" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="U4" s="30" t="n">
+      <c r="U4" s="31" t="n">
         <v>19</v>
       </c>
-      <c r="V4" s="30" t="n">
+      <c r="V4" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="W4" s="30" t="n">
+      <c r="W4" s="31" t="n">
         <v>21</v>
       </c>
-      <c r="X4" s="30" t="n">
+      <c r="X4" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="Y4" s="30" t="n">
+      <c r="Y4" s="31" t="n">
         <v>23</v>
       </c>
-      <c r="Z4" s="30" t="n">
+      <c r="Z4" s="31" t="n">
         <v>24</v>
       </c>
-      <c r="AA4" s="30" t="n">
+      <c r="AA4" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="AB4" s="30" t="n">
+      <c r="AB4" s="31" t="n">
         <v>26</v>
       </c>
-      <c r="AC4" s="30" t="n">
+      <c r="AC4" s="31" t="n">
         <v>27</v>
       </c>
-      <c r="AD4" s="30" t="n">
+      <c r="AD4" s="31" t="n">
         <v>28</v>
       </c>
-      <c r="AE4" s="30" t="n">
+      <c r="AE4" s="31" t="n">
         <v>29</v>
       </c>
-      <c r="AF4" s="30" t="n">
+      <c r="AF4" s="31" t="n">
         <v>30</v>
       </c>
-      <c r="AG4" s="30" t="n">
+      <c r="AG4" s="31" t="n">
         <v>31</v>
       </c>
-      <c r="AH4" s="30" t="n">
+      <c r="AH4" s="31" t="n">
         <v>32</v>
       </c>
-      <c r="AI4" s="30" t="n">
+      <c r="AI4" s="31" t="n">
         <v>33</v>
       </c>
-      <c r="AJ4" s="30" t="n">
+      <c r="AJ4" s="31" t="n">
         <v>34</v>
       </c>
-      <c r="AK4" s="30" t="n">
+      <c r="AK4" s="31" t="n">
         <v>35</v>
       </c>
-      <c r="AL4" s="30" t="n">
+      <c r="AL4" s="31" t="n">
         <v>36</v>
       </c>
     </row>
@@ -3818,147 +3832,147 @@
       <c r="A12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="32" t="n">
         <f aca="false">C9+C10+C11</f>
         <v>16387.5</v>
       </c>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="32" t="n">
         <f aca="false">D9+D10+D11</f>
         <v>16387.5</v>
       </c>
-      <c r="E12" s="31" t="n">
+      <c r="E12" s="32" t="n">
         <f aca="false">E9+E10+E11</f>
         <v>16387.5</v>
       </c>
-      <c r="F12" s="31" t="n">
+      <c r="F12" s="32" t="n">
         <f aca="false">F9+F10+F11</f>
         <v>16387.5</v>
       </c>
-      <c r="G12" s="31" t="n">
+      <c r="G12" s="32" t="n">
         <f aca="false">G9+G10+G11</f>
         <v>16387.5</v>
       </c>
-      <c r="H12" s="31" t="n">
+      <c r="H12" s="32" t="n">
         <f aca="false">H9+H10+H11</f>
         <v>16387.5</v>
       </c>
-      <c r="I12" s="31" t="n">
+      <c r="I12" s="32" t="n">
         <f aca="false">I9+I10+I11</f>
         <v>16387.5</v>
       </c>
-      <c r="J12" s="31" t="n">
+      <c r="J12" s="32" t="n">
         <f aca="false">J9+J10+J11</f>
         <v>16387.5</v>
       </c>
-      <c r="K12" s="31" t="n">
+      <c r="K12" s="32" t="n">
         <f aca="false">K9+K10+K11</f>
         <v>16387.5</v>
       </c>
-      <c r="L12" s="31" t="n">
+      <c r="L12" s="32" t="n">
         <f aca="false">L9+L10+L11</f>
         <v>16387.5</v>
       </c>
-      <c r="M12" s="31" t="n">
+      <c r="M12" s="32" t="n">
         <f aca="false">M9+M10+M11</f>
         <v>16387.5</v>
       </c>
-      <c r="N12" s="31" t="n">
+      <c r="N12" s="32" t="n">
         <f aca="false">N9+N10+N11</f>
         <v>16387.5</v>
       </c>
-      <c r="O12" s="31" t="n">
+      <c r="O12" s="32" t="n">
         <f aca="false">O9+O10+O11</f>
         <v>16879.125</v>
       </c>
-      <c r="P12" s="31" t="n">
+      <c r="P12" s="32" t="n">
         <f aca="false">P9+P10+P11</f>
         <v>16879.125</v>
       </c>
-      <c r="Q12" s="31" t="n">
+      <c r="Q12" s="32" t="n">
         <f aca="false">Q9+Q10+Q11</f>
         <v>16879.125</v>
       </c>
-      <c r="R12" s="31" t="n">
+      <c r="R12" s="32" t="n">
         <f aca="false">R9+R10+R11</f>
         <v>16879.125</v>
       </c>
-      <c r="S12" s="31" t="n">
+      <c r="S12" s="32" t="n">
         <f aca="false">S9+S10+S11</f>
         <v>16879.125</v>
       </c>
-      <c r="T12" s="31" t="n">
+      <c r="T12" s="32" t="n">
         <f aca="false">T9+T10+T11</f>
         <v>16879.125</v>
       </c>
-      <c r="U12" s="31" t="n">
+      <c r="U12" s="32" t="n">
         <f aca="false">U9+U10+U11</f>
         <v>16879.125</v>
       </c>
-      <c r="V12" s="31" t="n">
+      <c r="V12" s="32" t="n">
         <f aca="false">V9+V10+V11</f>
         <v>16879.125</v>
       </c>
-      <c r="W12" s="31" t="n">
+      <c r="W12" s="32" t="n">
         <f aca="false">W9+W10+W11</f>
         <v>16879.125</v>
       </c>
-      <c r="X12" s="31" t="n">
+      <c r="X12" s="32" t="n">
         <f aca="false">X9+X10+X11</f>
         <v>16879.125</v>
       </c>
-      <c r="Y12" s="31" t="n">
+      <c r="Y12" s="32" t="n">
         <f aca="false">Y9+Y10+Y11</f>
         <v>16879.125</v>
       </c>
-      <c r="Z12" s="31" t="n">
+      <c r="Z12" s="32" t="n">
         <f aca="false">Z9+Z10+Z11</f>
         <v>16879.125</v>
       </c>
-      <c r="AA12" s="31" t="n">
+      <c r="AA12" s="32" t="n">
         <f aca="false">AA9+AA10+AA11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AB12" s="31" t="n">
+      <c r="AB12" s="32" t="n">
         <f aca="false">AB9+AB10+AB11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AC12" s="31" t="n">
+      <c r="AC12" s="32" t="n">
         <f aca="false">AC9+AC10+AC11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AD12" s="31" t="n">
+      <c r="AD12" s="32" t="n">
         <f aca="false">AD9+AD10+AD11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AE12" s="31" t="n">
+      <c r="AE12" s="32" t="n">
         <f aca="false">AE9+AE10+AE11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AF12" s="31" t="n">
+      <c r="AF12" s="32" t="n">
         <f aca="false">AF9+AF10+AF11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AG12" s="31" t="n">
+      <c r="AG12" s="32" t="n">
         <f aca="false">AG9+AG10+AG11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AH12" s="31" t="n">
+      <c r="AH12" s="32" t="n">
         <f aca="false">AH9+AH10+AH11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AI12" s="31" t="n">
+      <c r="AI12" s="32" t="n">
         <f aca="false">AI9+AI10+AI11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AJ12" s="31" t="n">
+      <c r="AJ12" s="32" t="n">
         <f aca="false">AJ9+AJ10+AJ11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AK12" s="31" t="n">
+      <c r="AK12" s="32" t="n">
         <f aca="false">AK9+AK10+AK11</f>
         <v>17385.49875</v>
       </c>
-      <c r="AL12" s="31" t="n">
+      <c r="AL12" s="32" t="n">
         <f aca="false">AL9+AL10+AL11</f>
         <v>17385.49875</v>
       </c>
@@ -4434,147 +4448,147 @@
       <c r="A18" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="C18" s="32" t="n">
         <f aca="false">C12+C17</f>
         <v>14518.5</v>
       </c>
-      <c r="D18" s="31" t="n">
+      <c r="D18" s="32" t="n">
         <f aca="false">D12+D17</f>
         <v>14518.5</v>
       </c>
-      <c r="E18" s="31" t="n">
+      <c r="E18" s="32" t="n">
         <f aca="false">E12+E17</f>
         <v>14518.5</v>
       </c>
-      <c r="F18" s="31" t="n">
+      <c r="F18" s="32" t="n">
         <f aca="false">F12+F17</f>
         <v>14518.5</v>
       </c>
-      <c r="G18" s="31" t="n">
+      <c r="G18" s="32" t="n">
         <f aca="false">G12+G17</f>
         <v>14518.5</v>
       </c>
-      <c r="H18" s="31" t="n">
+      <c r="H18" s="32" t="n">
         <f aca="false">H12+H17</f>
         <v>14518.5</v>
       </c>
-      <c r="I18" s="31" t="n">
+      <c r="I18" s="32" t="n">
         <f aca="false">I12+I17</f>
         <v>14518.5</v>
       </c>
-      <c r="J18" s="31" t="n">
+      <c r="J18" s="32" t="n">
         <f aca="false">J12+J17</f>
         <v>14518.5</v>
       </c>
-      <c r="K18" s="31" t="n">
+      <c r="K18" s="32" t="n">
         <f aca="false">K12+K17</f>
         <v>14518.5</v>
       </c>
-      <c r="L18" s="31" t="n">
+      <c r="L18" s="32" t="n">
         <f aca="false">L12+L17</f>
         <v>14518.5</v>
       </c>
-      <c r="M18" s="31" t="n">
+      <c r="M18" s="32" t="n">
         <f aca="false">M12+M17</f>
         <v>14518.5</v>
       </c>
-      <c r="N18" s="31" t="n">
+      <c r="N18" s="32" t="n">
         <f aca="false">N12+N17</f>
         <v>14518.5</v>
       </c>
-      <c r="O18" s="31" t="n">
+      <c r="O18" s="32" t="n">
         <f aca="false">O12+O17</f>
         <v>14954.055</v>
       </c>
-      <c r="P18" s="31" t="n">
+      <c r="P18" s="32" t="n">
         <f aca="false">P12+P17</f>
         <v>14954.055</v>
       </c>
-      <c r="Q18" s="31" t="n">
+      <c r="Q18" s="32" t="n">
         <f aca="false">Q12+Q17</f>
         <v>14954.055</v>
       </c>
-      <c r="R18" s="31" t="n">
+      <c r="R18" s="32" t="n">
         <f aca="false">R12+R17</f>
         <v>14954.055</v>
       </c>
-      <c r="S18" s="31" t="n">
+      <c r="S18" s="32" t="n">
         <f aca="false">S12+S17</f>
         <v>14954.055</v>
       </c>
-      <c r="T18" s="31" t="n">
+      <c r="T18" s="32" t="n">
         <f aca="false">T12+T17</f>
         <v>14954.055</v>
       </c>
-      <c r="U18" s="31" t="n">
+      <c r="U18" s="32" t="n">
         <f aca="false">U12+U17</f>
         <v>14954.055</v>
       </c>
-      <c r="V18" s="31" t="n">
+      <c r="V18" s="32" t="n">
         <f aca="false">V12+V17</f>
         <v>14954.055</v>
       </c>
-      <c r="W18" s="31" t="n">
+      <c r="W18" s="32" t="n">
         <f aca="false">W12+W17</f>
         <v>14954.055</v>
       </c>
-      <c r="X18" s="31" t="n">
+      <c r="X18" s="32" t="n">
         <f aca="false">X12+X17</f>
         <v>14954.055</v>
       </c>
-      <c r="Y18" s="31" t="n">
+      <c r="Y18" s="32" t="n">
         <f aca="false">Y12+Y17</f>
         <v>14954.055</v>
       </c>
-      <c r="Z18" s="31" t="n">
+      <c r="Z18" s="32" t="n">
         <f aca="false">Z12+Z17</f>
         <v>14954.055</v>
       </c>
-      <c r="AA18" s="31" t="n">
+      <c r="AA18" s="32" t="n">
         <f aca="false">AA12+AA17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AB18" s="31" t="n">
+      <c r="AB18" s="32" t="n">
         <f aca="false">AB12+AB17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AC18" s="31" t="n">
+      <c r="AC18" s="32" t="n">
         <f aca="false">AC12+AC17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AD18" s="31" t="n">
+      <c r="AD18" s="32" t="n">
         <f aca="false">AD12+AD17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AE18" s="31" t="n">
+      <c r="AE18" s="32" t="n">
         <f aca="false">AE12+AE17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AF18" s="31" t="n">
+      <c r="AF18" s="32" t="n">
         <f aca="false">AF12+AF17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AG18" s="31" t="n">
+      <c r="AG18" s="32" t="n">
         <f aca="false">AG12+AG17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AH18" s="31" t="n">
+      <c r="AH18" s="32" t="n">
         <f aca="false">AH12+AH17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AI18" s="31" t="n">
+      <c r="AI18" s="32" t="n">
         <f aca="false">AI12+AI17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AJ18" s="31" t="n">
+      <c r="AJ18" s="32" t="n">
         <f aca="false">AJ12+AJ17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AK18" s="31" t="n">
+      <c r="AK18" s="32" t="n">
         <f aca="false">AK12+AK17</f>
         <v>15402.67665</v>
       </c>
-      <c r="AL18" s="31" t="n">
+      <c r="AL18" s="32" t="n">
         <f aca="false">AL12+AL17</f>
         <v>15402.67665</v>
       </c>
@@ -5199,147 +5213,147 @@
       <c r="A25" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C25" s="31" t="n">
+      <c r="C25" s="32" t="n">
         <f aca="false">C21+C22+C23+C24</f>
         <v>-4073.5</v>
       </c>
-      <c r="D25" s="31" t="n">
+      <c r="D25" s="32" t="n">
         <f aca="false">D21+D22+D23+D24</f>
         <v>-4073.5</v>
       </c>
-      <c r="E25" s="31" t="n">
+      <c r="E25" s="32" t="n">
         <f aca="false">E21+E22+E23+E24</f>
         <v>-4073.5</v>
       </c>
-      <c r="F25" s="31" t="n">
+      <c r="F25" s="32" t="n">
         <f aca="false">F21+F22+F23+F24</f>
         <v>-4073.5</v>
       </c>
-      <c r="G25" s="31" t="n">
+      <c r="G25" s="32" t="n">
         <f aca="false">G21+G22+G23+G24</f>
         <v>-4073.5</v>
       </c>
-      <c r="H25" s="31" t="n">
+      <c r="H25" s="32" t="n">
         <f aca="false">H21+H22+H23+H24</f>
         <v>-4073.5</v>
       </c>
-      <c r="I25" s="31" t="n">
+      <c r="I25" s="32" t="n">
         <f aca="false">I21+I22+I23+I24</f>
         <v>-4073.5</v>
       </c>
-      <c r="J25" s="31" t="n">
+      <c r="J25" s="32" t="n">
         <f aca="false">J21+J22+J23+J24</f>
         <v>-4073.5</v>
       </c>
-      <c r="K25" s="31" t="n">
+      <c r="K25" s="32" t="n">
         <f aca="false">K21+K22+K23+K24</f>
         <v>-4073.5</v>
       </c>
-      <c r="L25" s="31" t="n">
+      <c r="L25" s="32" t="n">
         <f aca="false">L21+L22+L23+L24</f>
         <v>-4073.5</v>
       </c>
-      <c r="M25" s="31" t="n">
+      <c r="M25" s="32" t="n">
         <f aca="false">M21+M22+M23+M24</f>
         <v>-4073.5</v>
       </c>
-      <c r="N25" s="31" t="n">
+      <c r="N25" s="32" t="n">
         <f aca="false">N21+N22+N23+N24</f>
         <v>-4073.5</v>
       </c>
-      <c r="O25" s="31" t="n">
+      <c r="O25" s="32" t="n">
         <f aca="false">O21+O22+O23+O24</f>
         <v>-4195.705</v>
       </c>
-      <c r="P25" s="31" t="n">
+      <c r="P25" s="32" t="n">
         <f aca="false">P21+P22+P23+P24</f>
         <v>-4195.705</v>
       </c>
-      <c r="Q25" s="31" t="n">
+      <c r="Q25" s="32" t="n">
         <f aca="false">Q21+Q22+Q23+Q24</f>
         <v>-4195.705</v>
       </c>
-      <c r="R25" s="31" t="n">
+      <c r="R25" s="32" t="n">
         <f aca="false">R21+R22+R23+R24</f>
         <v>-4195.705</v>
       </c>
-      <c r="S25" s="31" t="n">
+      <c r="S25" s="32" t="n">
         <f aca="false">S21+S22+S23+S24</f>
         <v>-4195.705</v>
       </c>
-      <c r="T25" s="31" t="n">
+      <c r="T25" s="32" t="n">
         <f aca="false">T21+T22+T23+T24</f>
         <v>-4195.705</v>
       </c>
-      <c r="U25" s="31" t="n">
+      <c r="U25" s="32" t="n">
         <f aca="false">U21+U22+U23+U24</f>
         <v>-4195.705</v>
       </c>
-      <c r="V25" s="31" t="n">
+      <c r="V25" s="32" t="n">
         <f aca="false">V21+V22+V23+V24</f>
         <v>-4195.705</v>
       </c>
-      <c r="W25" s="31" t="n">
+      <c r="W25" s="32" t="n">
         <f aca="false">W21+W22+W23+W24</f>
         <v>-4195.705</v>
       </c>
-      <c r="X25" s="31" t="n">
+      <c r="X25" s="32" t="n">
         <f aca="false">X21+X22+X23+X24</f>
         <v>-4195.705</v>
       </c>
-      <c r="Y25" s="31" t="n">
+      <c r="Y25" s="32" t="n">
         <f aca="false">Y21+Y22+Y23+Y24</f>
         <v>-4195.705</v>
       </c>
-      <c r="Z25" s="31" t="n">
+      <c r="Z25" s="32" t="n">
         <f aca="false">Z21+Z22+Z23+Z24</f>
         <v>-4195.705</v>
       </c>
-      <c r="AA25" s="31" t="n">
+      <c r="AA25" s="32" t="n">
         <f aca="false">AA21+AA22+AA23+AA24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AB25" s="31" t="n">
+      <c r="AB25" s="32" t="n">
         <f aca="false">AB21+AB22+AB23+AB24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AC25" s="31" t="n">
+      <c r="AC25" s="32" t="n">
         <f aca="false">AC21+AC22+AC23+AC24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AD25" s="31" t="n">
+      <c r="AD25" s="32" t="n">
         <f aca="false">AD21+AD22+AD23+AD24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AE25" s="31" t="n">
+      <c r="AE25" s="32" t="n">
         <f aca="false">AE21+AE22+AE23+AE24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AF25" s="31" t="n">
+      <c r="AF25" s="32" t="n">
         <f aca="false">AF21+AF22+AF23+AF24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AG25" s="31" t="n">
+      <c r="AG25" s="32" t="n">
         <f aca="false">AG21+AG22+AG23+AG24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AH25" s="31" t="n">
+      <c r="AH25" s="32" t="n">
         <f aca="false">AH21+AH22+AH23+AH24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AI25" s="31" t="n">
+      <c r="AI25" s="32" t="n">
         <f aca="false">AI21+AI22+AI23+AI24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AJ25" s="31" t="n">
+      <c r="AJ25" s="32" t="n">
         <f aca="false">AJ21+AJ22+AJ23+AJ24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AK25" s="31" t="n">
+      <c r="AK25" s="32" t="n">
         <f aca="false">AK21+AK22+AK23+AK24</f>
         <v>-4321.57615</v>
       </c>
-      <c r="AL25" s="31" t="n">
+      <c r="AL25" s="32" t="n">
         <f aca="false">AL21+AL22+AL23+AL24</f>
         <v>-4321.57615</v>
       </c>
@@ -5348,147 +5362,147 @@
       <c r="A26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="31" t="n">
+      <c r="C26" s="32" t="n">
         <f aca="false">C18+C25</f>
         <v>10445</v>
       </c>
-      <c r="D26" s="31" t="n">
+      <c r="D26" s="32" t="n">
         <f aca="false">D18+D25</f>
         <v>10445</v>
       </c>
-      <c r="E26" s="31" t="n">
+      <c r="E26" s="32" t="n">
         <f aca="false">E18+E25</f>
         <v>10445</v>
       </c>
-      <c r="F26" s="31" t="n">
+      <c r="F26" s="32" t="n">
         <f aca="false">F18+F25</f>
         <v>10445</v>
       </c>
-      <c r="G26" s="31" t="n">
+      <c r="G26" s="32" t="n">
         <f aca="false">G18+G25</f>
         <v>10445</v>
       </c>
-      <c r="H26" s="31" t="n">
+      <c r="H26" s="32" t="n">
         <f aca="false">H18+H25</f>
         <v>10445</v>
       </c>
-      <c r="I26" s="31" t="n">
+      <c r="I26" s="32" t="n">
         <f aca="false">I18+I25</f>
         <v>10445</v>
       </c>
-      <c r="J26" s="31" t="n">
+      <c r="J26" s="32" t="n">
         <f aca="false">J18+J25</f>
         <v>10445</v>
       </c>
-      <c r="K26" s="31" t="n">
+      <c r="K26" s="32" t="n">
         <f aca="false">K18+K25</f>
         <v>10445</v>
       </c>
-      <c r="L26" s="31" t="n">
+      <c r="L26" s="32" t="n">
         <f aca="false">L18+L25</f>
         <v>10445</v>
       </c>
-      <c r="M26" s="31" t="n">
+      <c r="M26" s="32" t="n">
         <f aca="false">M18+M25</f>
         <v>10445</v>
       </c>
-      <c r="N26" s="31" t="n">
+      <c r="N26" s="32" t="n">
         <f aca="false">N18+N25</f>
         <v>10445</v>
       </c>
-      <c r="O26" s="31" t="n">
+      <c r="O26" s="32" t="n">
         <f aca="false">O18+O25</f>
         <v>10758.35</v>
       </c>
-      <c r="P26" s="31" t="n">
+      <c r="P26" s="32" t="n">
         <f aca="false">P18+P25</f>
         <v>10758.35</v>
       </c>
-      <c r="Q26" s="31" t="n">
+      <c r="Q26" s="32" t="n">
         <f aca="false">Q18+Q25</f>
         <v>10758.35</v>
       </c>
-      <c r="R26" s="31" t="n">
+      <c r="R26" s="32" t="n">
         <f aca="false">R18+R25</f>
         <v>10758.35</v>
       </c>
-      <c r="S26" s="31" t="n">
+      <c r="S26" s="32" t="n">
         <f aca="false">S18+S25</f>
         <v>10758.35</v>
       </c>
-      <c r="T26" s="31" t="n">
+      <c r="T26" s="32" t="n">
         <f aca="false">T18+T25</f>
         <v>10758.35</v>
       </c>
-      <c r="U26" s="31" t="n">
+      <c r="U26" s="32" t="n">
         <f aca="false">U18+U25</f>
         <v>10758.35</v>
       </c>
-      <c r="V26" s="31" t="n">
+      <c r="V26" s="32" t="n">
         <f aca="false">V18+V25</f>
         <v>10758.35</v>
       </c>
-      <c r="W26" s="31" t="n">
+      <c r="W26" s="32" t="n">
         <f aca="false">W18+W25</f>
         <v>10758.35</v>
       </c>
-      <c r="X26" s="31" t="n">
+      <c r="X26" s="32" t="n">
         <f aca="false">X18+X25</f>
         <v>10758.35</v>
       </c>
-      <c r="Y26" s="31" t="n">
+      <c r="Y26" s="32" t="n">
         <f aca="false">Y18+Y25</f>
         <v>10758.35</v>
       </c>
-      <c r="Z26" s="31" t="n">
+      <c r="Z26" s="32" t="n">
         <f aca="false">Z18+Z25</f>
         <v>10758.35</v>
       </c>
-      <c r="AA26" s="31" t="n">
+      <c r="AA26" s="32" t="n">
         <f aca="false">AA18+AA25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AB26" s="31" t="n">
+      <c r="AB26" s="32" t="n">
         <f aca="false">AB18+AB25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AC26" s="31" t="n">
+      <c r="AC26" s="32" t="n">
         <f aca="false">AC18+AC25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AD26" s="31" t="n">
+      <c r="AD26" s="32" t="n">
         <f aca="false">AD18+AD25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AE26" s="31" t="n">
+      <c r="AE26" s="32" t="n">
         <f aca="false">AE18+AE25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AF26" s="31" t="n">
+      <c r="AF26" s="32" t="n">
         <f aca="false">AF18+AF25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AG26" s="31" t="n">
+      <c r="AG26" s="32" t="n">
         <f aca="false">AG18+AG25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AH26" s="31" t="n">
+      <c r="AH26" s="32" t="n">
         <f aca="false">AH18+AH25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AI26" s="31" t="n">
+      <c r="AI26" s="32" t="n">
         <f aca="false">AI18+AI25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AJ26" s="31" t="n">
+      <c r="AJ26" s="32" t="n">
         <f aca="false">AJ18+AJ25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AK26" s="31" t="n">
+      <c r="AK26" s="32" t="n">
         <f aca="false">AK18+AK25</f>
         <v>11081.1005</v>
       </c>
-      <c r="AL26" s="31" t="n">
+      <c r="AL26" s="32" t="n">
         <f aca="false">AL18+AL25</f>
         <v>11081.1005</v>
       </c>
@@ -5815,147 +5829,147 @@
       <c r="A31" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C31" s="31" t="n">
+      <c r="C31" s="32" t="n">
         <f aca="false">C29+C30</f>
         <v>-795.097736625515</v>
       </c>
-      <c r="D31" s="31" t="n">
+      <c r="D31" s="32" t="n">
         <f aca="false">D29+D30</f>
         <v>-790.121854193122</v>
       </c>
-      <c r="E31" s="31" t="n">
+      <c r="E31" s="32" t="n">
         <f aca="false">E29+E30</f>
         <v>-785.114142949681</v>
       </c>
-      <c r="F31" s="31" t="n">
+      <c r="F31" s="32" t="n">
         <f aca="false">F29+F30</f>
         <v>-780.07443048913</v>
       </c>
-      <c r="G31" s="31" t="n">
+      <c r="G31" s="32" t="n">
         <f aca="false">G29+G30</f>
         <v>-775.002543471544</v>
       </c>
-      <c r="H31" s="31" t="n">
+      <c r="H31" s="32" t="n">
         <f aca="false">H29+H30</f>
         <v>-769.898307618073</v>
       </c>
-      <c r="I31" s="31" t="n">
+      <c r="I31" s="32" t="n">
         <f aca="false">I29+I30</f>
         <v>-764.761547705854</v>
       </c>
-      <c r="J31" s="31" t="n">
+      <c r="J31" s="32" t="n">
         <f aca="false">J29+J30</f>
         <v>-759.592087562905</v>
       </c>
-      <c r="K31" s="31" t="n">
+      <c r="K31" s="32" t="n">
         <f aca="false">K29+K30</f>
         <v>-754.389750062974</v>
       </c>
-      <c r="L31" s="31" t="n">
+      <c r="L31" s="32" t="n">
         <f aca="false">L29+L30</f>
         <v>-749.154357120377</v>
       </c>
-      <c r="M31" s="31" t="n">
+      <c r="M31" s="32" t="n">
         <f aca="false">M29+M30</f>
         <v>-743.8857296848</v>
       </c>
-      <c r="N31" s="31" t="n">
+      <c r="N31" s="32" t="n">
         <f aca="false">N29+N30</f>
         <v>-738.583687736074</v>
       </c>
-      <c r="O31" s="31" t="n">
+      <c r="O31" s="32" t="n">
         <f aca="false">O29+O30</f>
         <v>-419.925056451759</v>
       </c>
-      <c r="P31" s="31" t="n">
+      <c r="P31" s="32" t="n">
         <f aca="false">P29+P30</f>
         <v>-414.582647683344</v>
       </c>
-      <c r="Q31" s="31" t="n">
+      <c r="Q31" s="32" t="n">
         <f aca="false">Q29+Q30</f>
         <v>-409.206278469456</v>
       </c>
-      <c r="R31" s="31" t="n">
+      <c r="R31" s="32" t="n">
         <f aca="false">R29+R30</f>
         <v>-403.795764857683</v>
       </c>
-      <c r="S31" s="31" t="n">
+      <c r="S31" s="32" t="n">
         <f aca="false">S29+S30</f>
         <v>-398.350921899203</v>
       </c>
-      <c r="T31" s="31" t="n">
+      <c r="T31" s="32" t="n">
         <f aca="false">T29+T30</f>
         <v>-392.871563643385</v>
       </c>
-      <c r="U31" s="31" t="n">
+      <c r="U31" s="32" t="n">
         <f aca="false">U29+U30</f>
         <v>-387.357503132375</v>
       </c>
-      <c r="V31" s="31" t="n">
+      <c r="V31" s="32" t="n">
         <f aca="false">V29+V30</f>
         <v>-381.808552395621</v>
       </c>
-      <c r="W31" s="31" t="n">
+      <c r="W31" s="32" t="n">
         <f aca="false">W29+W30</f>
         <v>-376.224522444397</v>
       </c>
-      <c r="X31" s="31" t="n">
+      <c r="X31" s="32" t="n">
         <f aca="false">X29+X30</f>
         <v>-370.605223266295</v>
       </c>
-      <c r="Y31" s="31" t="n">
+      <c r="Y31" s="32" t="n">
         <f aca="false">Y29+Y30</f>
         <v>-364.950463819669</v>
       </c>
-      <c r="Z31" s="31" t="n">
+      <c r="Z31" s="32" t="n">
         <f aca="false">Z29+Z30</f>
         <v>-359.260052028061</v>
       </c>
-      <c r="AA31" s="31" t="n">
+      <c r="AA31" s="32" t="n">
         <f aca="false">AA29+AA30</f>
         <v>-30.8111111326316</v>
       </c>
-      <c r="AB31" s="31" t="n">
+      <c r="AB31" s="32" t="n">
         <f aca="false">AB29+AB30</f>
         <v>-25.076630612436</v>
       </c>
-      <c r="AC31" s="31" t="n">
+      <c r="AC31" s="32" t="n">
         <f aca="false">AC29+AC30</f>
         <v>-19.3059152528394</v>
       </c>
-      <c r="AD31" s="31" t="n">
+      <c r="AD31" s="32" t="n">
         <f aca="false">AD29+AD30</f>
         <v>-13.4987687817975</v>
       </c>
-      <c r="AE31" s="31" t="n">
+      <c r="AE31" s="32" t="n">
         <f aca="false">AE29+AE30</f>
         <v>-7.65499386412012</v>
       </c>
-      <c r="AF31" s="31" t="n">
+      <c r="AF31" s="32" t="n">
         <f aca="false">AF29+AF30</f>
         <v>-1.77439209572185</v>
       </c>
-      <c r="AG31" s="31" t="n">
+      <c r="AG31" s="32" t="n">
         <f aca="false">AG29+AG30</f>
         <v>4.14323600216994</v>
       </c>
-      <c r="AH31" s="31" t="n">
+      <c r="AH31" s="32" t="n">
         <f aca="false">AH29+AH30</f>
         <v>10.0980909888422</v>
       </c>
-      <c r="AI31" s="31" t="n">
+      <c r="AI31" s="32" t="n">
         <f aca="false">AI29+AI30</f>
         <v>16.0903745099413</v>
       </c>
-      <c r="AJ31" s="31" t="n">
+      <c r="AJ31" s="32" t="n">
         <f aca="false">AJ29+AJ30</f>
         <v>22.1202893033624</v>
       </c>
-      <c r="AK31" s="31" t="n">
+      <c r="AK31" s="32" t="n">
         <f aca="false">AK29+AK30</f>
         <v>28.1880392051635</v>
       </c>
-      <c r="AL31" s="31" t="n">
+      <c r="AL31" s="32" t="n">
         <f aca="false">AL29+AL30</f>
         <v>34.2938291555147</v>
       </c>
@@ -6411,147 +6425,147 @@
       <c r="A35" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C35" s="31" t="n">
+      <c r="C35" s="32" t="n">
         <f aca="false">C31+C34</f>
         <v>-795.097736625515</v>
       </c>
-      <c r="D35" s="31" t="n">
+      <c r="D35" s="32" t="n">
         <f aca="false">D31+D34</f>
         <v>-790.121854193122</v>
       </c>
-      <c r="E35" s="31" t="n">
+      <c r="E35" s="32" t="n">
         <f aca="false">E31+E34</f>
         <v>-785.114142949681</v>
       </c>
-      <c r="F35" s="31" t="n">
+      <c r="F35" s="32" t="n">
         <f aca="false">F31+F34</f>
         <v>-780.07443048913</v>
       </c>
-      <c r="G35" s="31" t="n">
+      <c r="G35" s="32" t="n">
         <f aca="false">G31+G34</f>
         <v>-775.002543471544</v>
       </c>
-      <c r="H35" s="31" t="n">
+      <c r="H35" s="32" t="n">
         <f aca="false">H31+H34</f>
         <v>-769.898307618073</v>
       </c>
-      <c r="I35" s="31" t="n">
+      <c r="I35" s="32" t="n">
         <f aca="false">I31+I34</f>
         <v>-764.761547705854</v>
       </c>
-      <c r="J35" s="31" t="n">
+      <c r="J35" s="32" t="n">
         <f aca="false">J31+J34</f>
         <v>-759.592087562905</v>
       </c>
-      <c r="K35" s="31" t="n">
+      <c r="K35" s="32" t="n">
         <f aca="false">K31+K34</f>
         <v>-754.389750062974</v>
       </c>
-      <c r="L35" s="31" t="n">
+      <c r="L35" s="32" t="n">
         <f aca="false">L31+L34</f>
         <v>-749.154357120377</v>
       </c>
-      <c r="M35" s="31" t="n">
+      <c r="M35" s="32" t="n">
         <f aca="false">M31+M34</f>
         <v>-743.8857296848</v>
       </c>
-      <c r="N35" s="31" t="n">
+      <c r="N35" s="32" t="n">
         <f aca="false">N31+N34</f>
         <v>-738.583687736074</v>
       </c>
-      <c r="O35" s="31" t="n">
+      <c r="O35" s="32" t="n">
         <f aca="false">O31+O34</f>
         <v>-419.925056451759</v>
       </c>
-      <c r="P35" s="31" t="n">
+      <c r="P35" s="32" t="n">
         <f aca="false">P31+P34</f>
         <v>-414.582647683344</v>
       </c>
-      <c r="Q35" s="31" t="n">
+      <c r="Q35" s="32" t="n">
         <f aca="false">Q31+Q34</f>
         <v>-409.206278469456</v>
       </c>
-      <c r="R35" s="31" t="n">
+      <c r="R35" s="32" t="n">
         <f aca="false">R31+R34</f>
         <v>-403.795764857683</v>
       </c>
-      <c r="S35" s="31" t="n">
+      <c r="S35" s="32" t="n">
         <f aca="false">S31+S34</f>
         <v>-398.350921899203</v>
       </c>
-      <c r="T35" s="31" t="n">
+      <c r="T35" s="32" t="n">
         <f aca="false">T31+T34</f>
         <v>-392.871563643385</v>
       </c>
-      <c r="U35" s="31" t="n">
+      <c r="U35" s="32" t="n">
         <f aca="false">U31+U34</f>
         <v>-387.357503132375</v>
       </c>
-      <c r="V35" s="31" t="n">
+      <c r="V35" s="32" t="n">
         <f aca="false">V31+V34</f>
         <v>-381.808552395621</v>
       </c>
-      <c r="W35" s="31" t="n">
+      <c r="W35" s="32" t="n">
         <f aca="false">W31+W34</f>
         <v>-376.224522444397</v>
       </c>
-      <c r="X35" s="31" t="n">
+      <c r="X35" s="32" t="n">
         <f aca="false">X31+X34</f>
         <v>-370.605223266295</v>
       </c>
-      <c r="Y35" s="31" t="n">
+      <c r="Y35" s="32" t="n">
         <f aca="false">Y31+Y34</f>
         <v>-364.950463819669</v>
       </c>
-      <c r="Z35" s="31" t="n">
+      <c r="Z35" s="32" t="n">
         <f aca="false">Z31+Z34</f>
         <v>-359.260052028061</v>
       </c>
-      <c r="AA35" s="31" t="n">
+      <c r="AA35" s="32" t="n">
         <f aca="false">AA31+AA34</f>
         <v>-30.8111111326316</v>
       </c>
-      <c r="AB35" s="31" t="n">
+      <c r="AB35" s="32" t="n">
         <f aca="false">AB31+AB34</f>
         <v>-25.076630612436</v>
       </c>
-      <c r="AC35" s="31" t="n">
+      <c r="AC35" s="32" t="n">
         <f aca="false">AC31+AC34</f>
         <v>-19.3059152528394</v>
       </c>
-      <c r="AD35" s="31" t="n">
+      <c r="AD35" s="32" t="n">
         <f aca="false">AD31+AD34</f>
         <v>-13.4987687817975</v>
       </c>
-      <c r="AE35" s="31" t="n">
+      <c r="AE35" s="32" t="n">
         <f aca="false">AE31+AE34</f>
         <v>-7.65499386412012</v>
       </c>
-      <c r="AF35" s="31" t="n">
+      <c r="AF35" s="32" t="n">
         <f aca="false">AF31+AF34</f>
         <v>-1.77439209572185</v>
       </c>
-      <c r="AG35" s="31" t="n">
+      <c r="AG35" s="32" t="n">
         <f aca="false">AG31+AG34</f>
         <v>4.14323600216994</v>
       </c>
-      <c r="AH35" s="31" t="n">
+      <c r="AH35" s="32" t="n">
         <f aca="false">AH31+AH34</f>
         <v>10.0980909888422</v>
       </c>
-      <c r="AI35" s="31" t="n">
+      <c r="AI35" s="32" t="n">
         <f aca="false">AI31+AI34</f>
         <v>16.0903745099413</v>
       </c>
-      <c r="AJ35" s="31" t="n">
+      <c r="AJ35" s="32" t="n">
         <f aca="false">AJ31+AJ34</f>
         <v>22.1202893033624</v>
       </c>
-      <c r="AK35" s="31" t="n">
+      <c r="AK35" s="32" t="n">
         <f aca="false">AK31+AK34</f>
         <v>28.1880392051635</v>
       </c>
-      <c r="AL35" s="31" t="n">
+      <c r="AL35" s="32" t="n">
         <f aca="false">AL31+AL34</f>
         <v>34.2938291555147</v>
       </c>
@@ -10365,147 +10379,147 @@
       <c r="A69" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C69" s="31" t="n">
+      <c r="C69" s="32" t="n">
         <f aca="false">C65+C66+C68</f>
         <v>58003.0170514176</v>
       </c>
-      <c r="D69" s="31" t="n">
+      <c r="D69" s="32" t="n">
         <f aca="false">D65+D66+D68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="E69" s="31" t="n">
+      <c r="E69" s="32" t="n">
         <f aca="false">E65+E66+E68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="F69" s="31" t="n">
+      <c r="F69" s="32" t="n">
         <f aca="false">F65+F66+F68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="G69" s="31" t="n">
+      <c r="G69" s="32" t="n">
         <f aca="false">G65+G66+G68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="H69" s="31" t="n">
+      <c r="H69" s="32" t="n">
         <f aca="false">H65+H66+H68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="I69" s="31" t="n">
+      <c r="I69" s="32" t="n">
         <f aca="false">I65+I66+I68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="J69" s="31" t="n">
+      <c r="J69" s="32" t="n">
         <f aca="false">J65+J66+J68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="K69" s="31" t="n">
+      <c r="K69" s="32" t="n">
         <f aca="false">K65+K66+K68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="L69" s="31" t="n">
+      <c r="L69" s="32" t="n">
         <f aca="false">L65+L66+L68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="M69" s="31" t="n">
+      <c r="M69" s="32" t="n">
         <f aca="false">M65+M66+M68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="N69" s="31" t="n">
+      <c r="N69" s="32" t="n">
         <f aca="false">N65+N66+N68</f>
         <v>2568.51705141777</v>
       </c>
-      <c r="O69" s="31" t="n">
+      <c r="O69" s="32" t="n">
         <f aca="false">O65+O66+O68</f>
         <v>2901.15205141777</v>
       </c>
-      <c r="P69" s="31" t="n">
+      <c r="P69" s="32" t="n">
         <f aca="false">P65+P66+P68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="Q69" s="31" t="n">
+      <c r="Q69" s="32" t="n">
         <f aca="false">Q65+Q66+Q68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="R69" s="31" t="n">
+      <c r="R69" s="32" t="n">
         <f aca="false">R65+R66+R68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="S69" s="31" t="n">
+      <c r="S69" s="32" t="n">
         <f aca="false">S65+S66+S68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="T69" s="31" t="n">
+      <c r="T69" s="32" t="n">
         <f aca="false">T65+T66+T68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="U69" s="31" t="n">
+      <c r="U69" s="32" t="n">
         <f aca="false">U65+U66+U68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="V69" s="31" t="n">
+      <c r="V69" s="32" t="n">
         <f aca="false">V65+V66+V68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="W69" s="31" t="n">
+      <c r="W69" s="32" t="n">
         <f aca="false">W65+W66+W68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="X69" s="31" t="n">
+      <c r="X69" s="32" t="n">
         <f aca="false">X65+X66+X68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="Y69" s="31" t="n">
+      <c r="Y69" s="32" t="n">
         <f aca="false">Y65+Y66+Y68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="Z69" s="31" t="n">
+      <c r="Z69" s="32" t="n">
         <f aca="false">Z65+Z66+Z68</f>
         <v>2873.11705141777</v>
       </c>
-      <c r="AA69" s="31" t="n">
+      <c r="AA69" s="32" t="n">
         <f aca="false">AA65+AA66+AA68</f>
         <v>3215.73110141777</v>
       </c>
-      <c r="AB69" s="31" t="n">
+      <c r="AB69" s="32" t="n">
         <f aca="false">AB65+AB66+AB68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AC69" s="31" t="n">
+      <c r="AC69" s="32" t="n">
         <f aca="false">AC65+AC66+AC68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AD69" s="31" t="n">
+      <c r="AD69" s="32" t="n">
         <f aca="false">AD65+AD66+AD68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AE69" s="31" t="n">
+      <c r="AE69" s="32" t="n">
         <f aca="false">AE65+AE66+AE68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AF69" s="31" t="n">
+      <c r="AF69" s="32" t="n">
         <f aca="false">AF65+AF66+AF68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AG69" s="31" t="n">
+      <c r="AG69" s="32" t="n">
         <f aca="false">AG65+AG66+AG68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AH69" s="31" t="n">
+      <c r="AH69" s="32" t="n">
         <f aca="false">AH65+AH66+AH68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AI69" s="31" t="n">
+      <c r="AI69" s="32" t="n">
         <f aca="false">AI65+AI66+AI68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AJ69" s="31" t="n">
+      <c r="AJ69" s="32" t="n">
         <f aca="false">AJ65+AJ66+AJ68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AK69" s="31" t="n">
+      <c r="AK69" s="32" t="n">
         <f aca="false">AK65+AK66+AK68</f>
         <v>3186.85505141777</v>
       </c>
-      <c r="AL69" s="31" t="n">
+      <c r="AL69" s="32" t="n">
         <f aca="false">AL65+AL66+AL68</f>
         <v>3186.85505141777</v>
       </c>
@@ -10663,147 +10677,147 @@
       <c r="A71" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C71" s="31" t="n">
+      <c r="C71" s="32" t="n">
         <f aca="false">C70+C69</f>
         <v>58003.0170514176</v>
       </c>
-      <c r="D71" s="31" t="n">
+      <c r="D71" s="32" t="n">
         <f aca="false">D70+D69</f>
         <v>60571.5341028354</v>
       </c>
-      <c r="E71" s="31" t="n">
+      <c r="E71" s="32" t="n">
         <f aca="false">E70+E69</f>
         <v>63140.0511542531</v>
       </c>
-      <c r="F71" s="31" t="n">
+      <c r="F71" s="32" t="n">
         <f aca="false">F70+F69</f>
         <v>65708.5682056709</v>
       </c>
-      <c r="G71" s="31" t="n">
+      <c r="G71" s="32" t="n">
         <f aca="false">G70+G69</f>
         <v>68277.0852570887</v>
       </c>
-      <c r="H71" s="31" t="n">
+      <c r="H71" s="32" t="n">
         <f aca="false">H70+H69</f>
         <v>70845.6023085065</v>
       </c>
-      <c r="I71" s="31" t="n">
+      <c r="I71" s="32" t="n">
         <f aca="false">I70+I69</f>
         <v>73414.1193599242</v>
       </c>
-      <c r="J71" s="31" t="n">
+      <c r="J71" s="32" t="n">
         <f aca="false">J70+J69</f>
         <v>75982.636411342</v>
       </c>
-      <c r="K71" s="31" t="n">
+      <c r="K71" s="32" t="n">
         <f aca="false">K70+K69</f>
         <v>78551.1534627598</v>
       </c>
-      <c r="L71" s="31" t="n">
+      <c r="L71" s="32" t="n">
         <f aca="false">L70+L69</f>
         <v>81119.6705141776</v>
       </c>
-      <c r="M71" s="31" t="n">
+      <c r="M71" s="32" t="n">
         <f aca="false">M70+M69</f>
         <v>83688.1875655953</v>
       </c>
-      <c r="N71" s="31" t="n">
+      <c r="N71" s="32" t="n">
         <f aca="false">N70+N69</f>
         <v>86256.7046170131</v>
       </c>
-      <c r="O71" s="31" t="n">
+      <c r="O71" s="32" t="n">
         <f aca="false">O70+O69</f>
         <v>89157.8566684309</v>
       </c>
-      <c r="P71" s="31" t="n">
+      <c r="P71" s="32" t="n">
         <f aca="false">P70+P69</f>
         <v>92030.9737198486</v>
       </c>
-      <c r="Q71" s="31" t="n">
+      <c r="Q71" s="32" t="n">
         <f aca="false">Q70+Q69</f>
         <v>94904.0907712664</v>
       </c>
-      <c r="R71" s="31" t="n">
+      <c r="R71" s="32" t="n">
         <f aca="false">R70+R69</f>
         <v>97777.2078226842</v>
       </c>
-      <c r="S71" s="31" t="n">
+      <c r="S71" s="32" t="n">
         <f aca="false">S70+S69</f>
         <v>100650.324874102</v>
       </c>
-      <c r="T71" s="31" t="n">
+      <c r="T71" s="32" t="n">
         <f aca="false">T70+T69</f>
         <v>103523.44192552</v>
       </c>
-      <c r="U71" s="31" t="n">
+      <c r="U71" s="32" t="n">
         <f aca="false">U70+U69</f>
         <v>106396.558976937</v>
       </c>
-      <c r="V71" s="31" t="n">
+      <c r="V71" s="32" t="n">
         <f aca="false">V70+V69</f>
         <v>109269.676028355</v>
       </c>
-      <c r="W71" s="31" t="n">
+      <c r="W71" s="32" t="n">
         <f aca="false">W70+W69</f>
         <v>112142.793079773</v>
       </c>
-      <c r="X71" s="31" t="n">
+      <c r="X71" s="32" t="n">
         <f aca="false">X70+X69</f>
         <v>115015.910131191</v>
       </c>
-      <c r="Y71" s="31" t="n">
+      <c r="Y71" s="32" t="n">
         <f aca="false">Y70+Y69</f>
         <v>117889.027182609</v>
       </c>
-      <c r="Z71" s="31" t="n">
+      <c r="Z71" s="32" t="n">
         <f aca="false">Z70+Z69</f>
         <v>120762.144234026</v>
       </c>
-      <c r="AA71" s="31" t="n">
+      <c r="AA71" s="32" t="n">
         <f aca="false">AA70+AA69</f>
         <v>123977.875335444</v>
       </c>
-      <c r="AB71" s="31" t="n">
+      <c r="AB71" s="32" t="n">
         <f aca="false">AB70+AB69</f>
         <v>127164.730386862</v>
       </c>
-      <c r="AC71" s="31" t="n">
+      <c r="AC71" s="32" t="n">
         <f aca="false">AC70+AC69</f>
         <v>130351.58543828</v>
       </c>
-      <c r="AD71" s="31" t="n">
+      <c r="AD71" s="32" t="n">
         <f aca="false">AD70+AD69</f>
         <v>133538.440489697</v>
       </c>
-      <c r="AE71" s="31" t="n">
+      <c r="AE71" s="32" t="n">
         <f aca="false">AE70+AE69</f>
         <v>136725.295541115</v>
       </c>
-      <c r="AF71" s="31" t="n">
+      <c r="AF71" s="32" t="n">
         <f aca="false">AF70+AF69</f>
         <v>139912.150592533</v>
       </c>
-      <c r="AG71" s="31" t="n">
+      <c r="AG71" s="32" t="n">
         <f aca="false">AG70+AG69</f>
         <v>143099.005643951</v>
       </c>
-      <c r="AH71" s="31" t="n">
+      <c r="AH71" s="32" t="n">
         <f aca="false">AH70+AH69</f>
         <v>146285.860695368</v>
       </c>
-      <c r="AI71" s="31" t="n">
+      <c r="AI71" s="32" t="n">
         <f aca="false">AI70+AI69</f>
         <v>149472.715746786</v>
       </c>
-      <c r="AJ71" s="31" t="n">
+      <c r="AJ71" s="32" t="n">
         <f aca="false">AJ70+AJ69</f>
         <v>152659.570798204</v>
       </c>
-      <c r="AK71" s="31" t="n">
+      <c r="AK71" s="32" t="n">
         <f aca="false">AK70+AK69</f>
         <v>155846.425849622</v>
       </c>
-      <c r="AL71" s="31" t="n">
+      <c r="AL71" s="32" t="n">
         <f aca="false">AL70+AL69</f>
         <v>159033.28090104</v>
       </c>
@@ -10812,147 +10826,147 @@
       <c r="A72" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="C72" s="32" t="n">
+      <c r="C72" s="33" t="n">
         <f aca="false">IF(C26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="D72" s="32" t="n">
+      <c r="D72" s="33" t="n">
         <f aca="false">IF(D26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="E72" s="32" t="n">
+      <c r="E72" s="33" t="n">
         <f aca="false">IF(E26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="F72" s="32" t="n">
+      <c r="F72" s="33" t="n">
         <f aca="false">IF(F26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="G72" s="32" t="n">
+      <c r="G72" s="33" t="n">
         <f aca="false">IF(G26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="H72" s="32" t="n">
+      <c r="H72" s="33" t="n">
         <f aca="false">IF(H26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="I72" s="32" t="n">
+      <c r="I72" s="33" t="n">
         <f aca="false">IF(I26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="J72" s="32" t="n">
+      <c r="J72" s="33" t="n">
         <f aca="false">IF(J26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="K72" s="32" t="n">
+      <c r="K72" s="33" t="n">
         <f aca="false">IF(K26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="L72" s="32" t="n">
+      <c r="L72" s="33" t="n">
         <f aca="false">IF(L26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="M72" s="32" t="n">
+      <c r="M72" s="33" t="n">
         <f aca="false">IF(M26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="N72" s="32" t="n">
+      <c r="N72" s="33" t="n">
         <f aca="false">IF(N26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="O72" s="32" t="n">
+      <c r="O72" s="33" t="n">
         <f aca="false">IF(O26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="P72" s="32" t="n">
+      <c r="P72" s="33" t="n">
         <f aca="false">IF(P26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="Q72" s="32" t="n">
+      <c r="Q72" s="33" t="n">
         <f aca="false">IF(Q26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="R72" s="32" t="n">
+      <c r="R72" s="33" t="n">
         <f aca="false">IF(R26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="S72" s="32" t="n">
+      <c r="S72" s="33" t="n">
         <f aca="false">IF(S26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="T72" s="32" t="n">
+      <c r="T72" s="33" t="n">
         <f aca="false">IF(T26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="U72" s="32" t="n">
+      <c r="U72" s="33" t="n">
         <f aca="false">IF(U26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="V72" s="32" t="n">
+      <c r="V72" s="33" t="n">
         <f aca="false">IF(V26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="W72" s="32" t="n">
+      <c r="W72" s="33" t="n">
         <f aca="false">IF(W26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="X72" s="32" t="n">
+      <c r="X72" s="33" t="n">
         <f aca="false">IF(X26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="Y72" s="32" t="n">
+      <c r="Y72" s="33" t="n">
         <f aca="false">IF(Y26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="Z72" s="32" t="n">
+      <c r="Z72" s="33" t="n">
         <f aca="false">IF(Z26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AA72" s="32" t="n">
+      <c r="AA72" s="33" t="n">
         <f aca="false">IF(AA26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AB72" s="32" t="n">
+      <c r="AB72" s="33" t="n">
         <f aca="false">IF(AB26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AC72" s="32" t="n">
+      <c r="AC72" s="33" t="n">
         <f aca="false">IF(AC26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AD72" s="32" t="n">
+      <c r="AD72" s="33" t="n">
         <f aca="false">IF(AD26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AE72" s="32" t="n">
+      <c r="AE72" s="33" t="n">
         <f aca="false">IF(AE26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AF72" s="32" t="n">
+      <c r="AF72" s="33" t="n">
         <f aca="false">IF(AF26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AG72" s="32" t="n">
+      <c r="AG72" s="33" t="n">
         <f aca="false">IF(AG26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AH72" s="32" t="n">
+      <c r="AH72" s="33" t="n">
         <f aca="false">IF(AH26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AI72" s="32" t="n">
+      <c r="AI72" s="33" t="n">
         <f aca="false">IF(AI26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AJ72" s="32" t="n">
+      <c r="AJ72" s="33" t="n">
         <f aca="false">IF(AJ26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AK72" s="32" t="n">
+      <c r="AK72" s="33" t="n">
         <f aca="false">IF(AK26&gt;0,1,0)</f>
         <v>1</v>
       </c>
-      <c r="AL72" s="32" t="n">
+      <c r="AL72" s="33" t="n">
         <f aca="false">IF(AL26&gt;0,1,0)</f>
         <v>1</v>
       </c>
@@ -12119,15 +12133,15 @@
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$18:$AL$18)</f>
         <v>174222</v>
       </c>
-      <c r="C7" s="31" t="n">
+      <c r="C7" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$18:$AL$18)</f>
         <v>179448.66</v>
       </c>
-      <c r="D7" s="31" t="n">
+      <c r="D7" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$18:$AL$18)</f>
         <v>184832.1198</v>
       </c>
@@ -12221,15 +12235,15 @@
       <c r="A13" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B13" s="31" t="n">
+      <c r="B13" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$25:$AL$25)</f>
         <v>-48882</v>
       </c>
-      <c r="C13" s="31" t="n">
+      <c r="C13" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$25:$AL$25)</f>
         <v>-50348.46</v>
       </c>
-      <c r="D13" s="31" t="n">
+      <c r="D13" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$25:$AL$25)</f>
         <v>-51858.9138</v>
       </c>
@@ -12238,15 +12252,15 @@
       <c r="A14" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="31" t="n">
+      <c r="B14" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$26:$AL$26)</f>
         <v>125340</v>
       </c>
-      <c r="C14" s="31" t="n">
+      <c r="C14" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$26:$AL$26)</f>
         <v>129100.2</v>
       </c>
-      <c r="D14" s="31" t="n">
+      <c r="D14" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$26:$AL$26)</f>
         <v>132973.206</v>
       </c>
@@ -12323,15 +12337,15 @@
       <c r="A19" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="B19" s="33" t="n">
+      <c r="B19" s="34" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$31:$AL$31)</f>
         <v>-9205.67617522005</v>
       </c>
-      <c r="C19" s="33" t="n">
+      <c r="C19" s="34" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$31:$AL$31)</f>
         <v>-4678.93855009125</v>
       </c>
-      <c r="D19" s="33" t="n">
+      <c r="D19" s="34" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$31:$AL$31)</f>
         <v>16.8120474254474</v>
       </c>
@@ -12357,15 +12371,15 @@
       <c r="A21" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="31" t="n">
+      <c r="B21" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$35:$AL$35)</f>
         <v>-9205.67617522005</v>
       </c>
-      <c r="C21" s="31" t="n">
+      <c r="C21" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$35:$AL$35)</f>
         <v>-4678.93855009125</v>
       </c>
-      <c r="D21" s="31" t="n">
+      <c r="D21" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$35:$AL$35)</f>
         <v>16.8120474254474</v>
       </c>
@@ -12537,15 +12551,15 @@
       <c r="A10" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B10" s="31" t="n">
+      <c r="B10" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$65:$AL$65)</f>
         <v>48669.4102445331</v>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$65:$AL$65)</f>
         <v>52421.418980773</v>
       </c>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$65:$AL$65)</f>
         <v>57253.6988227342</v>
       </c>
@@ -12622,15 +12636,15 @@
       <c r="A15" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B15" s="31" t="n">
+      <c r="B15" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,B$3,Monthly!$C$68:$AL$68)</f>
         <v>1946587.29437248</v>
       </c>
-      <c r="C15" s="31" t="n">
+      <c r="C15" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,C$3,Monthly!$C$68:$AL$68)</f>
         <v>-14310.9793637598</v>
       </c>
-      <c r="D15" s="31" t="n">
+      <c r="D15" s="32" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,D$3,Monthly!$C$68:$AL$68)</f>
         <v>-15269.4121557209</v>
       </c>
@@ -12673,15 +12687,15 @@
       <c r="A18" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B18" s="31" t="n">
+      <c r="B18" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$71:$AL$71,B$3*12)</f>
         <v>86256.7046170131</v>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="C18" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$71:$AL$71,C$3*12)</f>
         <v>120762.144234026</v>
       </c>
-      <c r="D18" s="31" t="n">
+      <c r="D18" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$71:$AL$71,D$3*12)</f>
         <v>159033.28090104</v>
       </c>
@@ -12819,15 +12833,15 @@
       <c r="A9" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="B9" s="31" t="n">
+      <c r="B9" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$77:$AL$77,B$3*12)</f>
         <v>1938316.11819726</v>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$77:$AL$77,C$3*12)</f>
         <v>1919354.23528341</v>
       </c>
-      <c r="D9" s="31" t="n">
+      <c r="D9" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$77:$AL$77,D$3*12)</f>
         <v>1904130.51122512</v>
       </c>
@@ -12870,15 +12884,15 @@
       <c r="A12" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="B12" s="33" t="n">
+      <c r="B12" s="34" t="n">
         <f aca="false">INDEX(Monthly!$C$78:$AL$78,B$3*12)</f>
         <v>1187521.79437248</v>
       </c>
-      <c r="C12" s="33" t="n">
+      <c r="C12" s="34" t="n">
         <f aca="false">INDEX(Monthly!$C$78:$AL$78,C$3*12)</f>
         <v>1173238.85000872</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="34" t="n">
         <f aca="false">INDEX(Monthly!$C$78:$AL$78,D$3*12)</f>
         <v>1157998.313903</v>
       </c>
@@ -12921,15 +12935,15 @@
       <c r="A15" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="B15" s="33" t="n">
+      <c r="B15" s="34" t="n">
         <f aca="false">INDEX(Monthly!$C$79:$AL$79,B$3*12)</f>
         <v>750794.32382478</v>
       </c>
-      <c r="C15" s="33" t="n">
+      <c r="C15" s="34" t="n">
         <f aca="false">INDEX(Monthly!$C$79:$AL$79,C$3*12)</f>
         <v>746115.385274689</v>
       </c>
-      <c r="D15" s="33" t="n">
+      <c r="D15" s="34" t="n">
         <f aca="false">INDEX(Monthly!$C$79:$AL$79,D$3*12)</f>
         <v>746132.197322114</v>
       </c>
@@ -12938,15 +12952,15 @@
       <c r="A16" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="B16" s="31" t="n">
+      <c r="B16" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$80:$AL$80,B$3*12)</f>
         <v>1938316.11819726</v>
       </c>
-      <c r="C16" s="31" t="n">
+      <c r="C16" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$80:$AL$80,C$3*12)</f>
         <v>1919354.23528341</v>
       </c>
-      <c r="D16" s="31" t="n">
+      <c r="D16" s="32" t="n">
         <f aca="false">INDEX(Monthly!$C$80:$AL$80,D$3*12)</f>
         <v>1904130.51122511</v>
       </c>
@@ -13134,112 +13148,112 @@
       <c r="A4" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="C4" s="30" t="n">
+      <c r="C4" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="30" t="n">
+      <c r="D4" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="30" t="n">
+      <c r="E4" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="30" t="n">
+      <c r="F4" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="30" t="n">
+      <c r="G4" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="30" t="n">
+      <c r="H4" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="30" t="n">
+      <c r="I4" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="30" t="n">
+      <c r="J4" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="K4" s="30" t="n">
+      <c r="K4" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="L4" s="30" t="n">
+      <c r="L4" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="M4" s="30" t="n">
+      <c r="M4" s="31" t="n">
         <v>11</v>
       </c>
-      <c r="N4" s="30" t="n">
+      <c r="N4" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="O4" s="30" t="n">
+      <c r="O4" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="P4" s="30" t="n">
+      <c r="P4" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="Q4" s="30" t="n">
+      <c r="Q4" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="R4" s="30" t="n">
+      <c r="R4" s="31" t="n">
         <v>16</v>
       </c>
-      <c r="S4" s="30" t="n">
+      <c r="S4" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="T4" s="30" t="n">
+      <c r="T4" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="U4" s="30" t="n">
+      <c r="U4" s="31" t="n">
         <v>19</v>
       </c>
-      <c r="V4" s="30" t="n">
+      <c r="V4" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="W4" s="30" t="n">
+      <c r="W4" s="31" t="n">
         <v>21</v>
       </c>
-      <c r="X4" s="30" t="n">
+      <c r="X4" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="Y4" s="30" t="n">
+      <c r="Y4" s="31" t="n">
         <v>23</v>
       </c>
-      <c r="Z4" s="30" t="n">
+      <c r="Z4" s="31" t="n">
         <v>24</v>
       </c>
-      <c r="AA4" s="30" t="n">
+      <c r="AA4" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="AB4" s="30" t="n">
+      <c r="AB4" s="31" t="n">
         <v>26</v>
       </c>
-      <c r="AC4" s="30" t="n">
+      <c r="AC4" s="31" t="n">
         <v>27</v>
       </c>
-      <c r="AD4" s="30" t="n">
+      <c r="AD4" s="31" t="n">
         <v>28</v>
       </c>
-      <c r="AE4" s="30" t="n">
+      <c r="AE4" s="31" t="n">
         <v>29</v>
       </c>
-      <c r="AF4" s="30" t="n">
+      <c r="AF4" s="31" t="n">
         <v>30</v>
       </c>
-      <c r="AG4" s="30" t="n">
+      <c r="AG4" s="31" t="n">
         <v>31</v>
       </c>
-      <c r="AH4" s="30" t="n">
+      <c r="AH4" s="31" t="n">
         <v>32</v>
       </c>
-      <c r="AI4" s="30" t="n">
+      <c r="AI4" s="31" t="n">
         <v>33</v>
       </c>
-      <c r="AJ4" s="30" t="n">
+      <c r="AJ4" s="31" t="n">
         <v>34</v>
       </c>
-      <c r="AK4" s="30" t="n">
+      <c r="AK4" s="31" t="n">
         <v>35</v>
       </c>
-      <c r="AL4" s="30" t="n">
+      <c r="AL4" s="31" t="n">
         <v>36</v>
       </c>
     </row>
@@ -13396,147 +13410,147 @@
       <c r="A6" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="H6" s="34" t="n">
+      <c r="H6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I6" s="34" t="n">
+      <c r="I6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="J6" s="34" t="n">
+      <c r="J6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="K6" s="34" t="n">
+      <c r="K6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="L6" s="34" t="n">
+      <c r="L6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="M6" s="34" t="n">
+      <c r="M6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="N6" s="34" t="n">
+      <c r="N6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="O6" s="34" t="n">
+      <c r="O6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="P6" s="34" t="n">
+      <c r="P6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="34" t="n">
+      <c r="Q6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="R6" s="34" t="n">
+      <c r="R6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="S6" s="34" t="n">
+      <c r="S6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="T6" s="34" t="n">
+      <c r="T6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="U6" s="34" t="n">
+      <c r="U6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="V6" s="34" t="n">
+      <c r="V6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="W6" s="34" t="n">
+      <c r="W6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="X6" s="34" t="n">
+      <c r="X6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="34" t="n">
+      <c r="Y6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="34" t="n">
+      <c r="Z6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AA6" s="34" t="n">
+      <c r="AA6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AB6" s="34" t="n">
+      <c r="AB6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AC6" s="34" t="n">
+      <c r="AC6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AD6" s="34" t="n">
+      <c r="AD6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AE6" s="34" t="n">
+      <c r="AE6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AF6" s="34" t="n">
+      <c r="AF6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AG6" s="34" t="n">
+      <c r="AG6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AH6" s="34" t="n">
+      <c r="AH6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AI6" s="34" t="n">
+      <c r="AI6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AJ6" s="34" t="n">
+      <c r="AJ6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AK6" s="34" t="n">
+      <c r="AK6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AL6" s="34" t="n">
+      <c r="AL6" s="35" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
@@ -13545,147 +13559,147 @@
       <c r="A7" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C7" s="31" t="n">
+      <c r="C7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="D7" s="31" t="n">
+      <c r="D7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E7" s="31" t="n">
+      <c r="E7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F7" s="31" t="n">
+      <c r="F7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G7" s="31" t="n">
+      <c r="G7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="H7" s="31" t="n">
+      <c r="H7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I7" s="31" t="n">
+      <c r="I7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="J7" s="31" t="n">
+      <c r="J7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="K7" s="31" t="n">
+      <c r="K7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="L7" s="31" t="n">
+      <c r="L7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="M7" s="31" t="n">
+      <c r="M7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="N7" s="31" t="n">
+      <c r="N7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="O7" s="31" t="n">
+      <c r="O7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="P7" s="31" t="n">
+      <c r="P7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="Q7" s="31" t="n">
+      <c r="Q7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="R7" s="31" t="n">
+      <c r="R7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="S7" s="31" t="n">
+      <c r="S7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="T7" s="31" t="n">
+      <c r="T7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="U7" s="31" t="n">
+      <c r="U7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="V7" s="31" t="n">
+      <c r="V7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="W7" s="31" t="n">
+      <c r="W7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="X7" s="31" t="n">
+      <c r="X7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="Y7" s="31" t="n">
+      <c r="Y7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="Z7" s="31" t="n">
+      <c r="Z7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AA7" s="31" t="n">
+      <c r="AA7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AB7" s="31" t="n">
+      <c r="AB7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AC7" s="31" t="n">
+      <c r="AC7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AD7" s="31" t="n">
+      <c r="AD7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AE7" s="31" t="n">
+      <c r="AE7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AF7" s="31" t="n">
+      <c r="AF7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AG7" s="31" t="n">
+      <c r="AG7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AH7" s="31" t="n">
+      <c r="AH7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AI7" s="31" t="n">
+      <c r="AI7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AJ7" s="31" t="n">
+      <c r="AJ7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AK7" s="31" t="n">
+      <c r="AK7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="AL7" s="31" t="n">
+      <c r="AL7" s="32" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
@@ -13706,7 +13720,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -13767,7 +13781,7 @@
       <c r="A8" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B8" s="31" t="n">
+      <c r="B8" s="32" t="n">
         <f aca="false">B6+B7</f>
         <v>1905500</v>
       </c>
@@ -13826,19 +13840,19 @@
       <c r="A15" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="35" t="n">
+      <c r="B15" s="36" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="C15" s="35" t="n">
+      <c r="C15" s="36" t="n">
         <f aca="false">B15+1</f>
         <v>1</v>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="36" t="n">
         <f aca="false">C15+1</f>
         <v>2</v>
       </c>
-      <c r="E15" s="35" t="n">
+      <c r="E15" s="36" t="n">
         <f aca="false">D15+1</f>
         <v>3</v>
       </c>
@@ -13911,19 +13925,19 @@
         <v>214</v>
       </c>
       <c r="B19" s="19" t="n">
-        <f aca="false">IF(B$15=$E$15,$B$34,0)</f>
+        <f aca="false">IF(B$15=$E$15,$B$36,0)</f>
         <v>0</v>
       </c>
       <c r="C19" s="19" t="n">
-        <f aca="false">IF(C$15=$E$15,$B$34,0)</f>
+        <f aca="false">IF(C$15=$E$15,$B$36,0)</f>
         <v>0</v>
       </c>
       <c r="D19" s="19" t="n">
-        <f aca="false">IF(D$15=$E$15,$B$34,0)</f>
+        <f aca="false">IF(D$15=$E$15,$B$36,0)</f>
         <v>0</v>
       </c>
       <c r="E19" s="19" t="n">
-        <f aca="false">IF(E$15=$E$15,$B$34,0)</f>
+        <f aca="false">IF(E$15=$E$15,$B$36,0)</f>
         <v>1927618.99364444</v>
       </c>
     </row>
@@ -13931,19 +13945,19 @@
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="B20" s="31" t="n">
+      <c r="B20" s="32" t="n">
         <f aca="false">B16+B17+B18+B19</f>
         <v>-1905500</v>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C20" s="32" t="n">
         <f aca="false">C16+C17+C18+C19</f>
         <v>121840</v>
       </c>
-      <c r="D20" s="31" t="n">
+      <c r="D20" s="32" t="n">
         <f aca="false">D16+D17+D18+D19</f>
         <v>125495.2</v>
       </c>
-      <c r="E20" s="31" t="n">
+      <c r="E20" s="32" t="n">
         <f aca="false">E16+E17+E18+E19</f>
         <v>2056879.04964444</v>
       </c>
@@ -14016,19 +14030,19 @@
         <v>218</v>
       </c>
       <c r="B24" s="19" t="n">
-        <f aca="false">-IF(B$15=$E$15,$B$35,0)</f>
+        <f aca="false">-IF(B$15=$E$15,$B$37,0)</f>
         <v>-0</v>
       </c>
       <c r="C24" s="19" t="n">
-        <f aca="false">-IF(C$15=$E$15,$B$35,0)</f>
+        <f aca="false">-IF(C$15=$E$15,$B$37,0)</f>
         <v>-0</v>
       </c>
       <c r="D24" s="19" t="n">
-        <f aca="false">-IF(D$15=$E$15,$B$35,0)</f>
+        <f aca="false">-IF(D$15=$E$15,$B$37,0)</f>
         <v>-0</v>
       </c>
       <c r="E24" s="19" t="n">
-        <f aca="false">-IF(E$15=$E$15,$B$35,0)</f>
+        <f aca="false">-IF(E$15=$E$15,$B$37,0)</f>
         <v>-1157006.902853</v>
       </c>
     </row>
@@ -14036,19 +14050,19 @@
       <c r="A25" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="B25" s="31" t="n">
+      <c r="B25" s="32" t="n">
         <f aca="false">B20+B21+B22+B23+B24</f>
         <v>-705500</v>
       </c>
-      <c r="C25" s="31" t="n">
+      <c r="C25" s="32" t="n">
         <f aca="false">C20+C21+C22+C23+C24</f>
         <v>30822.2046170132</v>
       </c>
-      <c r="D25" s="31" t="n">
+      <c r="D25" s="32" t="n">
         <f aca="false">D20+D21+D22+D23+D24</f>
         <v>34477.4046170132</v>
       </c>
-      <c r="E25" s="31" t="n">
+      <c r="E25" s="32" t="n">
         <f aca="false">E20+E21+E22+E23+E24</f>
         <v>808854.351408458</v>
       </c>
@@ -14057,20 +14071,20 @@
       <c r="A26" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="36" t="str">
-        <f aca="false">IF(-(B22+B23)&gt;0,B17/-(B22+B23),"n/a")</f>
+      <c r="B26" s="37" t="str">
+        <f aca="false">IF(-(B22+B23)&gt;0.5,B17/-(B22+B23),"n/a")</f>
         <v>n/a</v>
       </c>
-      <c r="C26" s="36" t="n">
-        <f aca="false">IF(-(C22+C23)&gt;0,C17/-(C22+C23),"n/a")</f>
+      <c r="C26" s="37" t="n">
+        <f aca="false">IF(-(C22+C23)&gt;0.5,C17/-(C22+C23),"n/a")</f>
         <v>1.37709334172061</v>
       </c>
-      <c r="D26" s="36" t="n">
-        <f aca="false">IF(-(D22+D23)&gt;0,D17/-(D22+D23),"n/a")</f>
+      <c r="D26" s="37" t="n">
+        <f aca="false">IF(-(D22+D23)&gt;0.5,D17/-(D22+D23),"n/a")</f>
         <v>1.41840614197223</v>
       </c>
-      <c r="E26" s="36" t="n">
-        <f aca="false">IF(-(E22+E23)&gt;0,E17/-(E22+E23),"n/a")</f>
+      <c r="E26" s="37" t="n">
+        <f aca="false">IF(-(E22+E23)&gt;0.5,E17/-(E22+E23),"n/a")</f>
         <v>1.4609583262314</v>
       </c>
     </row>
@@ -14095,58 +14109,82 @@
         <v>0.0542058974018614</v>
       </c>
     </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="B28" s="36" t="n">
+        <f aca="false">SIGN(B20)</f>
+        <v>-1</v>
+      </c>
+      <c r="C28" s="36" t="n">
+        <f aca="false">IF(C20=0,B28,SIGN(C20))</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="36" t="n">
+        <f aca="false">IF(D20=0,C28,SIGN(D20))</f>
+        <v>1</v>
+      </c>
+      <c r="E28" s="36" t="n">
+        <f aca="false">IF(E20=0,D28,SIGN(E20))</f>
+        <v>1</v>
+      </c>
+    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
+      <c r="A29" s="11" t="s">
         <v>222</v>
       </c>
-      <c r="B30" s="19" t="n">
-        <f aca="false">E17*(1+Inputs!$E$14)</f>
-        <v>136962.40218</v>
+      <c r="B29" s="36" t="n">
+        <f aca="false">SIGN(B25)</f>
+        <v>-1</v>
+      </c>
+      <c r="C29" s="36" t="n">
+        <f aca="false">IF(C25=0,B29,SIGN(C25))</f>
+        <v>1</v>
+      </c>
+      <c r="D29" s="36" t="n">
+        <f aca="false">IF(D25=0,C29,SIGN(D25))</f>
+        <v>1</v>
+      </c>
+      <c r="E29" s="36" t="n">
+        <f aca="false">IF(E25=0,D29,SIGN(E25))</f>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="B31" s="12" t="n">
-        <f aca="false">Inputs!$E$29</f>
-        <v>0.0675</v>
-      </c>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
         <v>224</v>
       </c>
       <c r="B32" s="19" t="n">
-        <f aca="false">IF(B31&gt;0,B30/B31,0)</f>
-        <v>2029072.62488889</v>
+        <f aca="false">E17*(1+Inputs!$E$14)</f>
+        <v>136962.40218</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="B33" s="19" t="n">
-        <f aca="false">-B32*Inputs!$E$30</f>
-        <v>-101453.631244444</v>
+      <c r="B33" s="12" t="n">
+        <f aca="false">Inputs!$E$29</f>
+        <v>0.0675</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="B34" s="31" t="n">
-        <f aca="false">B32+B33</f>
-        <v>1927618.99364444</v>
+      <c r="B34" s="19" t="n">
+        <f aca="false">IF(B33&gt;0,B32/B33,0)</f>
+        <v>2029072.62488889</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14154,122 +14192,153 @@
         <v>227</v>
       </c>
       <c r="B35" s="19" t="n">
-        <f aca="false">INDEX(Monthly!$C$54:$AL$54,36)</f>
-        <v>1157006.902853</v>
+        <f aca="false">-B34*Inputs!$E$30</f>
+        <v>-101453.631244444</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="B36" s="15" t="n">
-        <f aca="false">B34-B35</f>
+      <c r="B36" s="32" t="n">
+        <f aca="false">B34+B35</f>
+        <v>1927618.99364444</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B37" s="19" t="n">
+        <f aca="false">INDEX(Monthly!$C$54:$AL$54,36)</f>
+        <v>1157006.902853</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B38" s="15" t="n">
+        <f aca="false">B36-B37</f>
         <v>770612.090791445</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="C39" s="9" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B40" s="20" t="n">
-        <f aca="false">IFERROR(IRR($B$20:$E$20,B41),IFERROR(IRR($B$20:$E$20),"n/a"))</f>
-        <v>0.0694044035752205</v>
-      </c>
-      <c r="C40" s="20" t="n">
-        <f aca="false">IFERROR(IRR($B$25:$E$25,C41),IFERROR(IRR($B$25:$E$25),"n/a"))</f>
-        <v>0.077168516706971</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="s">
+      <c r="C41" s="9" t="s">
         <v>233</v>
-      </c>
-      <c r="B41" s="20" t="n">
-        <f aca="false">IF(AND(SUMIF($B$20:$E$20,"&gt;0")&gt;0,-SUMIF($B$20:$E$20,"&lt;0")&gt;0),MAX(-0.99,(SUMIF($B$20:$E$20,"&gt;0")/(-SUMIF($B$20:$E$20,"&lt;0")))^(1/$E$15)-1),0.1)</f>
-        <v>0.0653802338076868</v>
-      </c>
-      <c r="C41" s="20" t="n">
-        <f aca="false">IF(AND(SUMIF($B$25:$E$25,"&gt;0")&gt;0,-SUMIF($B$25:$E$25,"&lt;0")&gt;0),MAX(-0.99,(SUMIF($B$25:$E$25,"&gt;0")/(-SUMIF($B$25:$E$25,"&lt;0")))^(1/$E$15)-1),0.1)</f>
-        <v>0.0740643549091244</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="B42" s="12" t="n">
-        <f aca="false">Inputs!$E$31</f>
-        <v>0.1</v>
+      <c r="B42" s="20" t="n">
+        <f aca="false">IF(B44=1,IFERROR(IRR($B$20:$E$20,B43),IFERROR(IRR($B$20:$E$20),"n/a")),"n/a")</f>
+        <v>0.0694044035752205</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <f aca="false">IF(C44=1,IFERROR(IRR($B$25:$E$25,C43),IFERROR(IRR($B$25:$E$25),"n/a")),"n/a")</f>
+        <v>0.077168516706971</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="B43" s="15" t="n">
-        <f aca="false">$B$20+NPV($B$42,$C$20:$E$20)</f>
-        <v>-145657.648651808</v>
-      </c>
-      <c r="C43" s="15" t="n">
-        <f aca="false">$B$25+NPV($B$42,$C$25:$E$25)</f>
-        <v>-41281.8451737355</v>
+      <c r="B43" s="20" t="n">
+        <f aca="false">IF(AND(SUMIF($B$20:$E$20,"&gt;0")&gt;0,-SUMIF($B$20:$E$20,"&lt;0")&gt;0),MAX(-0.99,(SUMIF($B$20:$E$20,"&gt;0")/(-SUMIF($B$20:$E$20,"&lt;0")))^(1/$E$15)-1),0.1)</f>
+        <v>0.0653802338076868</v>
+      </c>
+      <c r="C43" s="20" t="n">
+        <f aca="false">IF(AND(SUMIF($B$25:$E$25,"&gt;0")&gt;0,-SUMIF($B$25:$E$25,"&lt;0")&gt;0),MAX(-0.99,(SUMIF($B$25:$E$25,"&gt;0")/(-SUMIF($B$25:$E$25,"&lt;0")))^(1/$E$15)-1),0.1)</f>
+        <v>0.0740643549091244</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="B44" s="19" t="n">
-        <f aca="false">SUM($B$20:$E$20)</f>
-        <v>398714.249644444</v>
-      </c>
-      <c r="C44" s="19" t="n">
-        <f aca="false">SUM($B$25:$E$25)</f>
-        <v>168653.960642484</v>
+      <c r="B44" s="36" t="n">
+        <f aca="false">IF(AND(SUMPRODUCT(--($B$28:$D$28*$C$28:$E$28&lt;0))=1,SUMIF($B$20:$E$20,"&gt;0")&gt;=0.25*-SUMIF($B$20:$E$20,"&lt;0")),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="C44" s="36" t="n">
+        <f aca="false">IF(AND(SUMPRODUCT(--($B$29:$D$29*$C$29:$E$29&lt;0))=1,SUMIF($B$25:$E$25,"&gt;0")&gt;=0.25*-SUMIF($B$25:$E$25,"&lt;0")),1,0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="B45" s="36" t="n">
+      <c r="B45" s="12" t="n">
+        <f aca="false">Inputs!$E$31</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B46" s="15" t="n">
+        <f aca="false">$B$20+NPV($B$45,$C$20:$E$20)</f>
+        <v>-145657.648651808</v>
+      </c>
+      <c r="C46" s="15" t="n">
+        <f aca="false">$B$25+NPV($B$45,$C$25:$E$25)</f>
+        <v>-41281.8451737355</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B47" s="19" t="n">
+        <f aca="false">SUM($B$20:$E$20)</f>
+        <v>398714.249644444</v>
+      </c>
+      <c r="C47" s="19" t="n">
+        <f aca="false">SUM($B$25:$E$25)</f>
+        <v>168653.960642484</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="B48" s="37" t="n">
         <f aca="false">IF($B$20&lt;0,SUM($C$20:$E$20)/-$B$20,"n/a")</f>
         <v>1.20924389905245</v>
       </c>
-      <c r="C45" s="36" t="n">
+      <c r="C48" s="37" t="n">
         <f aca="false">IF($B$25&lt;0,SUM($C$25:$E$25)/-$B$25,"n/a")</f>
         <v>1.23905593287383</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11" t="s">
-        <v>238</v>
-      </c>
-      <c r="B46" s="20" t="n">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="B49" s="20" t="n">
         <f aca="false">IF(B6&gt;0,C17/B6,0)</f>
         <v>0.0677513513513514</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
-        <v>239</v>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -14305,229 +14374,229 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
-        <v>241</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>243</v>
+      <c r="A3" s="22" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B4" s="4" t="str">
         <f aca="false">IF(ABS(SUM('P&amp;L'!$B$5:$D$5)-SUM(Monthly!$C$12:$AL$12))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B5" s="4" t="str">
         <f aca="false">IF(ABS(SUM('P&amp;L'!$B$21:$D$21)-SUM(Monthly!$C$35:$AL$35))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B6" s="4" t="str">
         <f aca="false">IF(ABS(SUM(Monthly!$C$26:$AL$26)-SUM(Monthly!$C$18:$AL$18)-SUM(Monthly!$C$25:$AL$25))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B7" s="4" t="str">
         <f aca="false">IF(ABS(INDEX(Monthly!$C$71:$AL$71,36)-SUM(Monthly!$C$69:$AL$69))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B8" s="4" t="str">
         <f aca="false">IF(AND(ISNUMBER(Dashboard!B4),Dashboard!B4&gt;=1,Dashboard!B4&lt;=3,INT(Dashboard!B4)=Dashboard!B4),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B9" s="4" t="str">
         <f aca="false">IF(AND(Inputs!$B$9&gt;=Inputs!$C$9,Inputs!$C$9&gt;=Inputs!$D$9,Inputs!$B$13&lt;=Inputs!$C$13,Inputs!$C$13&lt;=Inputs!$D$13,Inputs!$B$14&lt;=Inputs!$C$14,Inputs!$C$14&lt;=Inputs!$D$14,Inputs!$B$15&gt;=Inputs!$C$15,Inputs!$C$15&gt;=Inputs!$D$15,Inputs!$B$16&lt;=Inputs!$C$16,Inputs!$C$16&lt;=Inputs!$D$16,Inputs!$B$19&gt;=Inputs!$C$19,Inputs!$C$19&gt;=Inputs!$D$19,Inputs!$B$23&gt;=Inputs!$C$23,Inputs!$C$23&gt;=Inputs!$D$23,Inputs!$B$25&gt;=Inputs!$C$25,Inputs!$C$25&gt;=Inputs!$D$25,Inputs!$B$29&gt;=Inputs!$C$29,Inputs!$C$29&gt;=Inputs!$D$29,Inputs!$B$30&gt;=Inputs!$C$30,Inputs!$C$30&gt;=Inputs!$D$30),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B10" s="4" t="str">
         <f aca="false">IF(AND(MIN('P&amp;L'!$B$8:$D$8)&gt;=0,MAX('P&amp;L'!$B$8:$D$8)&lt;=1),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B11" s="4" t="str">
         <f aca="false">IF(MIN(Monthly!$C$54:$AL$54)&gt;=-0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B12" s="4" t="str">
         <f aca="false">IF(ABS(SUM(Returns!$B$17:$E$17)-SUM(Monthly!$C$26:$AL$26))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B13" s="4" t="str">
         <f aca="false">IF(ABS(SUM(Returns!$B$16:$E$16)+SUM(Monthly!$C$38:$AL$38))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B14" s="4" t="str">
         <f aca="false">IF(ABS(SUM(Returns!$B$21:$E$21)+SUM(Returns!$B$23:$E$23)+SUM(Returns!$B$24:$E$24))&lt;0.5,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B15" s="4" t="str">
-        <f aca="false">IF(IF(ISNUMBER(Returns!B40),ABS(SUMPRODUCT(Returns!$B$20:$E$20/(1+Returns!B40)^Returns!$B$15:$E$15))&lt;1,TRUE()),"PASS","FAIL")</f>
+        <f aca="false">IF(IF(ISNUMBER(Returns!B42),ABS(SUMPRODUCT(Returns!$B$20:$E$20/(1+Returns!B42)^Returns!$B$15:$E$15))&lt;1,TRUE()),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B16" s="4" t="str">
-        <f aca="false">IF(IF(ISNUMBER(Returns!C40),ABS(SUMPRODUCT(Returns!$B$25:$E$25/(1+Returns!C40)^Returns!$B$15:$E$15))&lt;1,TRUE()),"PASS","FAIL")</f>
+        <f aca="false">IF(IF(ISNUMBER(Returns!C42),ABS(SUMPRODUCT(Returns!$B$25:$E$25/(1+Returns!C42)^Returns!$B$15:$E$15))&lt;1,TRUE()),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B17" s="4" t="str">
         <f aca="false">IF(SUMPRODUCT(--ISNUMBER(Returns!$C$26:$E$26),--(Returns!$C$26:$E$26&lt;1))=0,"PASS","WARN")</f>
         <v>PASS</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B18" s="4" t="str">
-        <f aca="false">IF(SUMPRODUCT(--ISERROR(Monthly!$C$4:$AL$81))+SUMPRODUCT(--ISERROR(Headcount!$C$4:$AL$7))+SUMPRODUCT(--ISERROR('P&amp;L'!$B$3:$D$22))+SUMPRODUCT(--ISERROR('Cash Flow'!$B$3:$D$18))+SUMPRODUCT(--ISERROR('Balance Sheet'!$B$3:$D$17))+SUMPRODUCT(--ISERROR(Dashboard!$B$25:$D$40))+SUMPRODUCT(--ISERROR(Returns!$A$3:$E$48))=0,"PASS","FAIL")</f>
+        <f aca="false">IF(SUMPRODUCT(--ISERROR(Monthly!$C$4:$AL$81))+SUMPRODUCT(--ISERROR(Headcount!$C$4:$AL$7))+SUMPRODUCT(--ISERROR('P&amp;L'!$B$3:$D$22))+SUMPRODUCT(--ISERROR('Cash Flow'!$B$3:$D$18))+SUMPRODUCT(--ISERROR('Balance Sheet'!$B$3:$D$17))+SUMPRODUCT(--ISERROR(Dashboard!$B$25:$D$40))+SUMPRODUCT(--ISERROR(Returns!$A$3:$E$51))=0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B19" s="4" t="str">
         <f aca="false">IF(SUMPRODUCT(--(ABS(Monthly!$C$81:$AL$81)&gt;0.5))=0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B20" s="4" t="str">
         <f aca="false">IF(MIN(Monthly!$C$71:$AL$71)&gt;=0,"PASS","WARN")</f>
         <v>PASS</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="B22" s="37" t="str">
+        <v>281</v>
+      </c>
+      <c r="B22" s="38" t="str">
         <f aca="false">IF(COUNTIF(B4:B20,"FAIL")&gt;0,"FAIL",IF(COUNTIF(B4:B20,"WARN")&gt;0,"PASS WITH WARNINGS","PASS"))</f>
         <v>PASS</v>
       </c>

</xml_diff>